<commit_message>
feat: restore node-node-battle daily flow
</commit_message>
<xml_diff>
--- a/xlsx/ysbzs_master.xlsx
+++ b/xlsx/ysbzs_master.xlsx
@@ -13,9 +13,6 @@
     <sheet name="SHOP_ITEMS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="MECHANISMS" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="TRIALS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SHAPE_CATALOG" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="QUALITY_GROWTH" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="QUALITY_UPGRADES" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PETS'!$A$1:$L$128</definedName>
@@ -23,9 +20,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'SHOP_ITEMS'!$A$1:$H$128</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MECHANISMS'!$A$1:$H$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TRIALS'!$A$1:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SHAPE_CATALOG'!$A$1:$H$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'QUALITY_GROWTH'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'QUALITY_UPGRADES'!$A$1:$I$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8603,7 +8597,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -8618,7 +8612,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>98.7</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -8653,7 +8647,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -8668,7 +8662,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>150.1</t>
+          <t>108.6</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -8703,7 +8697,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -8718,7 +8712,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>202.7</t>
+          <t>146.7</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -8753,7 +8747,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -8768,7 +8762,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>256.7</t>
+          <t>185.7</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -8803,7 +8797,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -8818,7 +8812,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>311.8</t>
+          <t>225.6</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -8853,7 +8847,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -8868,7 +8862,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>98.7</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -8903,7 +8897,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -8918,7 +8912,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>150.1</t>
+          <t>108.6</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -8953,7 +8947,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -8968,7 +8962,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>202.7</t>
+          <t>146.7</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -9003,7 +8997,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -9018,7 +9012,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>256.7</t>
+          <t>185.7</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -9053,7 +9047,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -9068,7 +9062,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>311.8</t>
+          <t>225.6</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -23810,4403 +23804,4 @@
   <autoFilter ref="A1:I10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>shape_id</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>group</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>cell_count</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>settle_count</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>offsets</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>grid</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>形状01</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":1}]</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>....... / ...●■.. / .......</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>一格，右侧相邻。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>形状02</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>....... / ...●.■. / .......</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>一格，右侧隔一格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>形状03</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":3}]</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>....... / ...●..■ / .......</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>一格，右侧隔两格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>形状04</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":4}]</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>........ / ...●...■ / ........</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>一格，右侧更远点。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>形状05</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":1},{"dr":0,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>....... / ...●■■. / .......</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>二格，右侧连续两格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>形状06</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":-1},{"dr":0,"dc":1}]</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>....... / ..■●■.. / .......</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>二格，角色左右各一格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>形状07</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":-2},{"dr":0,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>....... / .■.●.■. / .......</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>二格，角色左右隔点。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>形状08</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":2},{"dr":0,"dc":3}]</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>....... / ...●.■■ / .......</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>二格，右侧远端连续两格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>形状09</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":1},{"dr":1,"dc":1}]</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>....■.. / ...●... / ....■..</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>二格，右上与右下。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>形状10</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":2},{"dr":1,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>.....■. / ...●... / .....■.</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>二格，隔点右上与右下。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>形状11</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":-1},{"dr":1,"dc":1}]</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>..■.... / ...●... / ....■..</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>二格，左上与右下对角。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>two</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>形状12</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":-1},{"dr":0,"dc":3}]</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>....... / ..■●...■ / .......</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>二格，左邻一格与右侧远点。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>形状13</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":1},{"dr":0,"dc":1},{"dr":1,"dc":1}]</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>....■.. / ...●■.. / ....■..</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>三格，右侧相邻竖三格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>形状14</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":2},{"dr":0,"dc":1},{"dr":1,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>.....■. / ...●■.. / .....■.</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>三格，右侧近点加远端上下。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>形状15</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":0,"dc":1},{"dr":0,"dc":2},{"dr":0,"dc":3}]</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>....... / ...●■■■ / .......</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>三格，右侧连续三格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>形状16</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":2},{"dr":0,"dc":2},{"dr":1,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>.....■. / ...●.■. / .....■.</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>三格，隔点竖三格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>形状17</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":0},{"dr":0,"dc":1},{"dr":1,"dc":0}]</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>...■... / ...●■.. / ...■...</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>三格，上下夹身加右侧相邻。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>形状18</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":0},{"dr":-1,"dc":1},{"dr":0,"dc":1}]</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>...■■.. / ...●■.. / .......</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>三格，右上小角。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>three</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>形状19</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>[{"dr":-1,"dc":1},{"dr":-1,"dc":2},{"dr":0,"dc":2}]</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>....■■. / ...●.■. / .......</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>三格，隔点右上小角。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H20"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>quality</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>shape_size</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>hp_bonus</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>atk_bonus</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>mechanic</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>bronze</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>青铜</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>基础</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>只有基础生命、攻击和 3 个行动形状。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>bronze</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>青铜</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>基础</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>只有基础生命、攻击和 3 个行动形状。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>bronze</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>青铜</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>基础</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>只有基础生命、攻击和 3 个行动形状。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>白银</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>白银 Buff</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>获得小幅数值成长，并获得 1 个自动触发的白银 Buff。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>白银</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>白银 Buff</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>获得小幅数值成长，并获得 1 个自动触发的白银 Buff。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>白银</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>白银 Buff</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>获得小幅数值成长，并获得 1 个自动触发的白银 Buff。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>黄金</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>黄金升级</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>获得中幅数值成长，并获得 1 个黄金升级。黄金升级主要围绕形状强化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>黄金</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>黄金升级</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>获得中幅数值成长，并获得 1 个黄金升级。黄金升级主要围绕形状强化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>黄金</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>黄金升级</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>获得中幅数值成长，并获得 1 个黄金升级。黄金升级主要围绕形状强化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>钻石</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>钻石质变</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>获得高幅数值成长，并获得 1 个钻石质变。钻石主要改变形状、结算或棋盘。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>钻石</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>钻石质变</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>获得高幅数值成长，并获得 1 个钻石质变。钻石主要改变形状、结算或棋盘。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>钻石</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>钻石质变</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>获得高幅数值成长，并获得 1 个钻石质变。钻石主要改变形状、结算或棋盘。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G13"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I69"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>upgrade_id</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>quality</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>operation_level</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>allowed_shape_sizes</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>effect</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>design_note</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>runtime_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>护体</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>回合开始时，获得 15 点护盾。</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>S02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>自愈</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>回合开始时，恢复自身 20 点生命值。</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>S03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>壮体</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>回合开始时，最大生命值翻倍，但最大生命值最多不超过 30。</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>S04</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>元素回响</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>造成元素伤害时，该元素伤害重复结算 1 次。</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>S05</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>收尾暴击</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>2|3</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>本次行动的最后一击必定暴击。</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>更适合二格、三格、多段结算角色。</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>S06</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>连击倍增</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>2|3</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>第一击伤害减半，之后每一击都是前一击的 2 倍。</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>S07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>越战越勇</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>每击杀 5 个怪，永久 +1 攻击力。</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>S08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>本命爆发</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>silver</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>passive</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>如果自身携带和自己相同的元素，元素爆发翻倍。</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>G01</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>攻守切换</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>dualMode</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>每回合可在攻/守之间切换。攻形态伤害 +2；守形态回合开始获得 8 护盾。</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>G02</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>稳爆切换</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>dualMode</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>可在稳定/爆发之间切换。稳定形态攻击 +1；爆发形态本回合第一次命中伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>金色核心格</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>每个行动形状中有 1 个金色核心格，核心格命中敌人时伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>G04</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>守护核心格</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>核心格覆盖友方时，该友方获得 8 护盾。</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>G05</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>回春核心格</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>核心格覆盖友方时，恢复 6 生命。</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>G06</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>破敌核心格</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>核心格命中敌人时，额外造成 2 点破甲伤害。</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>G07</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>正向强化</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>形状朝向正前方的最远格伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>背向守势</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>形状背后的格子若覆盖友方，该友方获得 10 护盾。</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>G09</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>左右借势</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>2|3</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>形状左右两侧格命中敌人时，各额外造成 1 点伤害。</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>G10</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>终点重击</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>形状最远端格子命中敌人时，伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>G11</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>单挑</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>如果本次形状只命中 1 个敌人，伤害 +5。</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>G12</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>点穴</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>命中敌人后，使该敌人下次受到伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>G13</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>隔山打牛</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>隔点形状命中时，伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>G14</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>破绽一击</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>dualMode</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>可切换稳击/重击。稳击伤害 +2；重击伤害 +6，但本回合只能结算这一个形状格。</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>G15</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>斩首</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>如果目标生命值不高于 8，额外造成 8 点伤害。</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>G16</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>追魂点</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>若该格击杀敌人，对最近敌人追加 3 点伤害。</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>精准印记</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>manualMark</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>每回合可选择自己 1 个作用格，使其获得印记。该格本回合伤害 +5。</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>手动选格，数量要少。只给一格英雄比较安全。</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>G18</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>双点连击</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>如果两个作用格都命中敌人，第二个命中的敌人伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>G19</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>前后夹击</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>前后两个格子都命中敌人时，两个敌人各额外受到 2 点伤害。</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>G20</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>对角穿心</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>对角两格命中时，较远的目标伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>G21</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>一攻一守</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>dualMode</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>两格中靠前格伤害 +2；靠后格若覆盖友方，则该友方获得 8 护盾。</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>G22</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>双印择一</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>manualMark</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>每回合可在两个作用格中选择 1 格加金印。命中敌人伤害 +4；覆盖友方护盾 +8。</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>二格英雄可少量使用，不能泛滥。</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>G23</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>连环标记</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>第一个命中的敌人被标记，第二个命中的敌人伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>G24</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>双锋</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>dualMode</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>可切换同伤/主副。同伤为两个格子各 +1 伤害；主副为第一个格子 +4，第二个格子不加成。</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>G25</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>三格核心</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>三格形状中固定 1 个核心格，核心格伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>G26</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>横扫压制</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>横扫三格命中 2 个以上敌人时，每个敌人额外受到 1 点伤害。</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>G27</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>竖线贯通</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>直线三格从近到远结算，第三格伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>G28</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>三点成阵</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>empoweredCell</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>三个作用格都覆盖到单位时，敌人受伤 +2，友方获得 5 护盾。</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>G29</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>首尾呼应</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>directionBonus</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>形状第一格和最远格同时命中时，最远格伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>G30</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>三选一金印</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>gold</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>manualMark</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>每回合可从三个作用格中选 1 个加金印。该格伤害 +3。</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>三格本身覆盖大，所以手动强化数值要比一格、二格低。</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>末端延伸</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>形状最远端额外延伸 1 格。</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>D02</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>起点回扫</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>2|3</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>形状结算后，反方向再结算 1 次，反向伤害 -2。</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>D03</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>镜像形状</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>1|2</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>当前形状会向相反方向复制 1 次。</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>不建议给三格，容易爆表。</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>D04</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>斜向复制</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>1|2</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>当前形状命中后，在斜向相邻位置额外生成 1 个作用格。</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>核心扩散</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>命中目标后，对目标上下左右各造成 1 点溅射伤害。</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>D06</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>双端开花</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>两个作用格的外侧各额外延伸 1 格，但额外格伤害 -2。</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>三格收束</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>三格形状如果只命中 1 个敌人，该敌人额外受到 6 点伤害。</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>D08</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>三格外放</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>三格形状命中 2 个以上敌人时，额外对每个目标造成 2 点伤害。</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>角形补点</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>L 型三格的缺角位置额外生成 1 个作用格，伤害 -2。</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>直线贯穿</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>shapeMutation</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>直线形状末端再贯穿 1 格，额外格伤害 -1。</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr"/>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>抢先结算</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>该角色总是最先结算。</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>D12</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>压轴结算</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>该角色总是最后结算，最后一击伤害 +5。</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>残血追击</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>若本次结算后有敌人生命不高于 5，对其追加 5 点伤害。</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr"/>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>D14</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>击杀连锁</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>1|2</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>击杀敌人后，对最近敌人追加 4 点伤害。</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr"/>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>D15</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>破阵启动</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>若本次命中 3 个单位，立即额外结算一次核心格。</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>D16</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>反复敲打</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>如果只命中 1 个敌人，同一格重复结算 1 次。</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>D17</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>二段行动</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>本角色先结算一半伤害，所有友方结算后再结算剩余伤害。</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>有一定理解成本，建议少量使用。</t>
-        </is>
-      </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>D18</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>元素先爆</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>如果本次触发元素爆发，该元素爆发提前到本角色普通伤害前结算。</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>D19</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>收割顺序</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>结算时优先攻击生命最低的目标。</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>会改变默认结算逻辑，建议只给少数角色。</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>D20</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>反向结算</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>settlementMutation</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>2|3</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>形状从最远格开始结算，而不是从近格开始结算。</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr"/>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>D21</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>火痕</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>形状覆盖过的空格留下火痕 1 回合，敌人站上受到 3 点火伤害。</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr"/>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>D22</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>水痕</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下水痕 1 回合，友方站上恢复 5 生命。</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr"/>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>D23</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>风痕</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下风痕 1 回合，友方站上时下次伤害 +2。</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr"/>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>D24</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>土痕</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下土痕 1 回合，友方站上获得 8 护盾。</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr"/>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>D25</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>金痕</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下金痕 1 回合，下一次命中该格敌人的攻击伤害 +2。</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr"/>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>D26</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>木痕</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下木痕 1 回合，回合开始时恢复站在上面的友方 4 生命。</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr"/>
-      <c r="I65" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>D27</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>佛光</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下佛光 1 回合，友方站上恢复 6 生命，敌人站上无效果。</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr"/>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>D28</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>流沙</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下流沙 1 回合，敌人站上受到 2 点伤害，并使其下次受伤 +2。</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr"/>
-      <c r="I67" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>D29</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>妖印</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>覆盖格留下妖印 1 回合，敌人站上后被标记，下次受到伤害 +4。</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr"/>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>D30</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>纸符</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>diamond</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>boardTrace</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>1|2|3</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>核心格留下纸符 1 回合，下一次经过该格的作用形状额外结算 1 次。</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>最有纸上西游特色，但强度较高，建议稀有。</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>implemented</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I69"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: close June 30 gameplay batch
</commit_message>
<xml_diff>
--- a/xlsx/ysbzs_master.xlsx
+++ b/xlsx/ysbzs_master.xlsx
@@ -12338,7 +12338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="8" min="1" max="1"/>
@@ -13328,6 +13328,33 @@
       <c r="E40" t="inlineStr">
         <is>
           <t>已存在</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>商店公开价目</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>青铜=2；白银=4；黄金=6；钻石=8</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>商店价格和售卖规则使用玩家可见品质轴，pT 只做内部池等级</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>已对齐</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>导出 06_shop_rewards.csv 时写入 默认价/价格覆盖</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: split enemy movement and attack counts
</commit_message>
<xml_diff>
--- a/xlsx/ysbzs_master.xlsx
+++ b/xlsx/ysbzs_master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9e3cb3f1ff6448c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETS" sheetId="2" r:id="R4d6f21ab74bd4950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_STORES" sheetId="3" r:id="R9a580a19bc6a4c97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WAVES" sheetId="4" r:id="Rc398ff0c5a294abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_ITEMS" sheetId="5" r:id="R0855529b36454ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MECHANICS_QUALITY" sheetId="6" r:id="R353bfe98a8b74e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHAPES_TRIALS" sheetId="7" r:id="Ref83b74f5ab24d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re7eceb7b832f450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETS" sheetId="2" r:id="Ra1eb943d9d754779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_STORES" sheetId="3" r:id="R833c300e42894194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WAVES" sheetId="4" r:id="R5bcedc693a75436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_ITEMS" sheetId="5" r:id="R25b622b63d934f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MECHANICS_QUALITY" sheetId="6" r:id="R54beb1d6afcf4723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHAPES_TRIALS" sheetId="7" r:id="R8ffabded54c14aef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +36,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -63,14 +63,54 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E5F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E5F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF9DC3E6"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
@@ -109,6 +149,47 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -531,7 +612,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R440bbd410913489d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf17097e533494565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -553,6 +634,8 @@
     <x:col min="11" max="11" width="26" customWidth="1"/>
     <x:col min="12" max="12" width="18" customWidth="1"/>
     <x:col min="13" max="13" width="26" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -595,6 +678,12 @@
       <x:c r="M1" s="2" t="str">
         <x:v>note</x:v>
       </x:c>
+      <x:c r="N1" s="29" t="str">
+        <x:v>enemy_move_range</x:v>
+      </x:c>
+      <x:c r="O1" s="29" t="str">
+        <x:v>enemy_attack_count</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
@@ -634,6 +723,12 @@
       <x:c r="M2" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N2" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O2" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
@@ -673,6 +768,12 @@
       <x:c r="M3" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N3" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O3" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="str">
@@ -712,6 +813,12 @@
       <x:c r="M4" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N4" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O4" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
@@ -751,6 +858,12 @@
       <x:c r="M5" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N5" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O5" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
@@ -790,6 +903,12 @@
       <x:c r="M6" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N6" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O6" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="str">
@@ -829,6 +948,12 @@
       <x:c r="M7" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N7" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O7" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="str">
@@ -868,6 +993,12 @@
       <x:c r="M8" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；前7个进入重新定位：已清空定位并重置为无机制。</x:v>
       </x:c>
+      <x:c r="N8" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O8" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="str">
@@ -909,6 +1040,12 @@
       <x:c r="M9" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；第8-12批按前7个青铜基准重平衡。</x:v>
       </x:c>
+      <x:c r="N9" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O9" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="3" t="str">
@@ -950,6 +1087,12 @@
       <x:c r="M10" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；第8-12批按前7个青铜基准重平衡。</x:v>
       </x:c>
+      <x:c r="N10" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O10" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="3" t="str">
@@ -991,6 +1134,12 @@
       <x:c r="M11" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；第8-12批按前7个青铜基准重平衡。</x:v>
       </x:c>
+      <x:c r="N11" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O11" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="3" t="str">
@@ -1032,6 +1181,12 @@
       <x:c r="M12" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；第8-12批按前7个青铜基准重平衡。</x:v>
       </x:c>
+      <x:c r="N12" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O12" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="3" t="str">
@@ -1073,6 +1228,12 @@
       <x:c r="M13" s="3" t="str">
         <x:v>旧定位=牵制；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。；第8-12批按前7个青铜基准重平衡。</x:v>
       </x:c>
+      <x:c r="N13" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O13" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="3" t="str">
@@ -1114,6 +1275,12 @@
       <x:c r="M14" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N14" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O14" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="3" t="str">
@@ -1155,6 +1322,12 @@
       <x:c r="M15" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N15" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O15" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="3" t="str">
@@ -1196,6 +1369,12 @@
       <x:c r="M16" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N16" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O16" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="3" t="str">
@@ -1237,6 +1416,12 @@
       <x:c r="M17" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N17" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O17" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="3" t="str">
@@ -1278,6 +1463,12 @@
       <x:c r="M18" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N18" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O18" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="3" t="str">
@@ -1319,6 +1510,12 @@
       <x:c r="M19" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N19" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O19" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="3" t="str">
@@ -1360,6 +1557,12 @@
       <x:c r="M20" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N20" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O20" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="3" t="str">
@@ -1401,6 +1604,12 @@
       <x:c r="M21" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N21" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O21" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="3" t="str">
@@ -1442,6 +1651,12 @@
       <x:c r="M22" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N22" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O22" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="3" t="str">
@@ -1483,6 +1698,12 @@
       <x:c r="M23" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N23" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O23" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="3" t="str">
@@ -1524,6 +1745,12 @@
       <x:c r="M24" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N24" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O24" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="3" t="str">
@@ -1565,6 +1792,12 @@
       <x:c r="M25" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N25" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O25" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="3" t="str">
@@ -1606,6 +1839,12 @@
       <x:c r="M26" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N26" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O26" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="3" t="str">
@@ -1647,6 +1886,12 @@
       <x:c r="M27" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N27" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O27" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="3" t="str">
@@ -1688,6 +1933,12 @@
       <x:c r="M28" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N28" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O28" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="3" t="str">
@@ -1729,6 +1980,12 @@
       <x:c r="M29" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N29" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O29" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="3" t="str">
@@ -1770,6 +2027,12 @@
       <x:c r="M30" s="3" t="str">
         <x:v>经济补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N30" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O30" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="3" t="str">
@@ -1811,6 +2074,12 @@
       <x:c r="M31" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N31" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O31" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="3" t="str">
@@ -1852,6 +2121,12 @@
       <x:c r="M32" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N32" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O32" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="3" t="str">
@@ -1893,6 +2168,12 @@
       <x:c r="M33" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N33" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O33" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="3" t="str">
@@ -1934,6 +2215,12 @@
       <x:c r="M34" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N34" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O34" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="3" t="str">
@@ -1975,6 +2262,12 @@
       <x:c r="M35" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N35" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O35" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="3" t="str">
@@ -2016,6 +2309,12 @@
       <x:c r="M36" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N36" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O36" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="3" t="str">
@@ -2057,6 +2356,12 @@
       <x:c r="M37" s="3" t="str">
         <x:v>经济补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N37" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O37" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="3" t="str">
@@ -2098,6 +2403,12 @@
       <x:c r="M38" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N38" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O38" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="3" t="str">
@@ -2139,6 +2450,12 @@
       <x:c r="M39" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N39" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O39" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="3" t="str">
@@ -2180,6 +2497,12 @@
       <x:c r="M40" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N40" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O40" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="3" t="str">
@@ -2221,6 +2544,12 @@
       <x:c r="M41" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N41" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O41" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="3" t="str">
@@ -2262,6 +2591,12 @@
       <x:c r="M42" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N42" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O42" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="3" t="str">
@@ -2303,6 +2638,12 @@
       <x:c r="M43" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N43" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O43" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="3" t="str">
@@ -2344,6 +2685,12 @@
       <x:c r="M44" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N44" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O44" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="3" t="str">
@@ -2385,6 +2732,12 @@
       <x:c r="M45" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N45" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O45" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="3" t="str">
@@ -2426,6 +2779,12 @@
       <x:c r="M46" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N46" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O46" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="3" t="str">
@@ -2467,6 +2826,12 @@
       <x:c r="M47" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N47" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O47" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="3" t="str">
@@ -2508,6 +2873,12 @@
       <x:c r="M48" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N48" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O48" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="3" t="str">
@@ -2549,6 +2920,12 @@
       <x:c r="M49" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N49" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O49" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="3" t="str">
@@ -2590,6 +2967,12 @@
       <x:c r="M50" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N50" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O50" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="3" t="str">
@@ -2631,6 +3014,12 @@
       <x:c r="M51" s="3" t="str">
         <x:v>召唤补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N51" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O51" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="3" t="str">
@@ -2672,6 +3061,12 @@
       <x:c r="M52" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N52" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O52" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="3" t="str">
@@ -2713,6 +3108,12 @@
       <x:c r="M53" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N53" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O53" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="3" t="str">
@@ -2754,6 +3155,12 @@
       <x:c r="M54" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N54" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O54" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="3" t="str">
@@ -2795,6 +3202,12 @@
       <x:c r="M55" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N55" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O55" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="3" t="str">
@@ -2836,6 +3249,12 @@
       <x:c r="M56" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N56" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O56" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="3" t="str">
@@ -2877,6 +3296,12 @@
       <x:c r="M57" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N57" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O57" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="3" t="str">
@@ -2918,6 +3343,12 @@
       <x:c r="M58" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N58" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O58" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="3" t="str">
@@ -2959,6 +3390,12 @@
       <x:c r="M59" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N59" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O59" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="3" t="str">
@@ -3000,6 +3437,12 @@
       <x:c r="M60" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N60" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O60" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="3" t="str">
@@ -3041,6 +3484,12 @@
       <x:c r="M61" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N61" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O61" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="3" t="str">
@@ -3082,6 +3531,12 @@
       <x:c r="M62" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N62" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O62" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="3" t="str">
@@ -3123,6 +3578,12 @@
       <x:c r="M63" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N63" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O63" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="3" t="str">
@@ -3164,6 +3625,12 @@
       <x:c r="M64" s="3" t="str">
         <x:v>召唤补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N64" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O64" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="3" t="str">
@@ -3205,6 +3672,12 @@
       <x:c r="M65" s="3" t="str">
         <x:v>召唤补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N65" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O65" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="3" t="str">
@@ -3246,6 +3719,12 @@
       <x:c r="M66" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N66" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O66" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="3" t="str">
@@ -3287,6 +3766,12 @@
       <x:c r="M67" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N67" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O67" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="3" t="str">
@@ -3328,6 +3813,12 @@
       <x:c r="M68" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N68" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O68" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="3" t="str">
@@ -3369,6 +3860,12 @@
       <x:c r="M69" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N69" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O69" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="3" t="str">
@@ -3410,6 +3907,12 @@
       <x:c r="M70" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N70" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O70" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="3" t="str">
@@ -3451,6 +3954,12 @@
       <x:c r="M71" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N71" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O71" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="3" t="str">
@@ -3492,6 +4001,12 @@
       <x:c r="M72" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N72" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O72" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="3" t="str">
@@ -3533,6 +4048,12 @@
       <x:c r="M73" s="3" t="str">
         <x:v>召唤补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N73" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O73" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="3" t="str">
@@ -3574,6 +4095,12 @@
       <x:c r="M74" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N74" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O74" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="3" t="str">
@@ -3615,6 +4142,12 @@
       <x:c r="M75" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N75" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O75" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="3" t="str">
@@ -3656,6 +4189,12 @@
       <x:c r="M76" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N76" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O76" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="3" t="str">
@@ -3697,6 +4236,12 @@
       <x:c r="M77" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N77" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O77" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="3" t="str">
@@ -3738,6 +4283,12 @@
       <x:c r="M78" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N78" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O78" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="3" t="str">
@@ -3779,6 +4330,12 @@
       <x:c r="M79" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N79" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O79" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="3" t="str">
@@ -3820,6 +4377,12 @@
       <x:c r="M80" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N80" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O80" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="3" t="str">
@@ -3861,6 +4424,12 @@
       <x:c r="M81" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N81" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O81" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="3" t="str">
@@ -3902,6 +4471,12 @@
       <x:c r="M82" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N82" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O82" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="3" t="str">
@@ -3943,6 +4518,12 @@
       <x:c r="M83" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N83" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O83" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="3" t="str">
@@ -3984,6 +4565,12 @@
       <x:c r="M84" s="3" t="str">
         <x:v>召唤补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N84" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O84" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="3" t="str">
@@ -4025,6 +4612,12 @@
       <x:c r="M85" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N85" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O85" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="3" t="str">
@@ -4066,6 +4659,12 @@
       <x:c r="M86" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N86" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O86" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="3" t="str">
@@ -4107,6 +4706,12 @@
       <x:c r="M87" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N87" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O87" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="3" t="str">
@@ -4148,6 +4753,12 @@
       <x:c r="M88" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N88" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O88" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="3" t="str">
@@ -4189,6 +4800,12 @@
       <x:c r="M89" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N89" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O89" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="3" t="str">
@@ -4230,6 +4847,12 @@
       <x:c r="M90" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N90" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O90" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="3" t="str">
@@ -4271,6 +4894,12 @@
       <x:c r="M91" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N91" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O91" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="3" t="str">
@@ -4312,6 +4941,12 @@
       <x:c r="M92" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N92" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O92" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="3" t="str">
@@ -4353,6 +4988,12 @@
       <x:c r="M93" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N93" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O93" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="3" t="str">
@@ -4394,6 +5035,12 @@
       <x:c r="M94" s="3" t="str">
         <x:v>召唤补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N94" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O94" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="3" t="str">
@@ -4435,6 +5082,12 @@
       <x:c r="M95" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N95" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O95" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="3" t="str">
@@ -4476,6 +5129,12 @@
       <x:c r="M96" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N96" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O96" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="3" t="str">
@@ -4517,6 +5176,12 @@
       <x:c r="M97" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N97" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O97" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="3" t="str">
@@ -4558,6 +5223,12 @@
       <x:c r="M98" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N98" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O98" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="3" t="str">
@@ -4599,6 +5270,12 @@
       <x:c r="M99" s="3" t="str">
         <x:v>经济补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N99" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O99" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="3" t="str">
@@ -4640,6 +5317,12 @@
       <x:c r="M100" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N100" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O100" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="3" t="str">
@@ -4681,6 +5364,12 @@
       <x:c r="M101" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N101" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O101" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="3" t="str">
@@ -4722,6 +5411,12 @@
       <x:c r="M102" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N102" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O102" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="3" t="str">
@@ -4763,6 +5458,12 @@
       <x:c r="M103" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N103" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O103" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="3" t="str">
@@ -4804,6 +5505,12 @@
       <x:c r="M104" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N104" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O104" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="3" t="str">
@@ -4845,6 +5552,12 @@
       <x:c r="M105" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N105" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O105" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="3" t="str">
@@ -4886,6 +5599,12 @@
       <x:c r="M106" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N106" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O106" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="3" t="str">
@@ -4927,6 +5646,12 @@
       <x:c r="M107" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N107" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O107" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="3" t="str">
@@ -4968,6 +5693,12 @@
       <x:c r="M108" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N108" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O108" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="3" t="str">
@@ -5009,6 +5740,12 @@
       <x:c r="M109" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N109" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O109" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="3" t="str">
@@ -5050,6 +5787,12 @@
       <x:c r="M110" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N110" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O110" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="3" t="str">
@@ -5091,6 +5834,12 @@
       <x:c r="M111" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N111" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O111" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="3" t="str">
@@ -5132,6 +5881,12 @@
       <x:c r="M112" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N112" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O112" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="3" t="str">
@@ -5173,6 +5928,12 @@
       <x:c r="M113" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N113" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O113" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="3" t="str">
@@ -5214,6 +5975,12 @@
       <x:c r="M114" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N114" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O114" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="3" t="str">
@@ -5255,6 +6022,12 @@
       <x:c r="M115" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N115" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O115" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="3" t="str">
@@ -5296,6 +6069,12 @@
       <x:c r="M116" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N116" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O116" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="3" t="str">
@@ -5337,6 +6116,12 @@
       <x:c r="M117" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N117" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O117" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="3" t="str">
@@ -5378,6 +6163,12 @@
       <x:c r="M118" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N118" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O118" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="3" t="str">
@@ -5419,6 +6210,12 @@
       <x:c r="M119" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N119" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O119" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="3" t="str">
@@ -5460,6 +6257,12 @@
       <x:c r="M120" s="3" t="str">
         <x:v>治疗补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N120" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O120" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="3" t="str">
@@ -5501,6 +6304,12 @@
       <x:c r="M121" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N121" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O121" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="3" t="str">
@@ -5542,6 +6351,12 @@
       <x:c r="M122" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N122" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O122" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="3" t="str">
@@ -5583,6 +6398,12 @@
       <x:c r="M123" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N123" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O123" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="3" t="str">
@@ -5624,6 +6445,12 @@
       <x:c r="M124" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N124" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O124" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="3" t="str">
@@ -5665,6 +6492,12 @@
       <x:c r="M125" s="3" t="str">
         <x:v>旧定位=防御；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N125" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O125" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="3" t="str">
@@ -5706,6 +6539,12 @@
       <x:c r="M126" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N126" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O126" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="3" t="str">
@@ -5747,6 +6586,12 @@
       <x:c r="M127" s="3" t="str">
         <x:v>旧定位=牵制；控制补预算；基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N127" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O127" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="3" t="str">
@@ -5788,11 +6633,23 @@
       <x:c r="M128" s="3" t="str">
         <x:v>基础字段按原 PETS 表恢复；正式19形状与机制接入保持当前版本。</x:v>
       </x:c>
+      <x:c r="N128" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O128" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="whole" operator="between" sqref="N2:O128">
+      <x:formula1>0</x:formula1>
+      <x:formula2>99</x:formula2>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd141c21c28ae4585"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3be4c4067e704147"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6917,7 +7774,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R257dbe8f46f64b3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f85110635454e08"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
data: add Journey shops with six-pet minimum
</commit_message>
<xml_diff>
--- a/xlsx/ysbzs_master.xlsx
+++ b/xlsx/ysbzs_master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re7eceb7b832f450d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETS" sheetId="2" r:id="Ra1eb943d9d754779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_STORES" sheetId="3" r:id="R833c300e42894194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WAVES" sheetId="4" r:id="R5bcedc693a75436e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_ITEMS" sheetId="5" r:id="R25b622b63d934f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MECHANICS_QUALITY" sheetId="6" r:id="R54beb1d6afcf4723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHAPES_TRIALS" sheetId="7" r:id="R8ffabded54c14aef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6d85dd06fd254d69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETS" sheetId="2" r:id="R26d7d55025bb47b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_STORES" sheetId="3" r:id="Re009305e4059458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WAVES" sheetId="4" r:id="R2170680bb9e041d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHOP_ITEMS" sheetId="5" r:id="Rd60e7ebf59f24ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MECHANICS_QUALITY" sheetId="6" r:id="R677f45f23b5345e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHAPES_TRIALS" sheetId="7" r:id="Ra2a4bd1a8ac8461c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ShopStoresTable" displayName="ShopStoresTable" ref="A1:I38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I38"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ShopStoresTable" displayName="ShopStoresTable" ref="A1:I80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I80"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="shop_store_id"/>
     <x:tableColumn id="2" name="name"/>
@@ -598,7 +598,7 @@
         <x:v>元素规则</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>帕鲁九系：无、火、水、草、雷、冰、地、暗、龙；element 单元格用顿号保留双属性，商品会进入全部对应元素店。</x:v>
+        <x:v>帕鲁九系：无、火、水、草、雷、冰、地、暗、龙；element 单元格用顿号保留双属性，商品会进入全部对应元素店。 西游化语义：无=凡兽、火=丹火、水=江河、草=灵木、雷=天雷、冰=寒霜、地=厚土、暗=阴煞、龙=龙脉。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -612,7 +612,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf17097e533494565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6545c57d78840d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -690,7 +690,7 @@
         <x:v>pal_001</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>棉悠悠</x:v>
+        <x:v>棉角羊</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
         <x:v>无</x:v>
@@ -700,7 +700,7 @@
       </x:c>
       <x:c r="E2" s="3"/>
       <x:c r="F2" s="3" t="str">
-        <x:v>night_base, elem_无, tier_pT1</x:v>
+        <x:v>night_base, elem_无, tier_pT1, shop_store_37, shop_store_55, shop_store_73</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
         <x:v>21</x:v>
@@ -735,7 +735,7 @@
         <x:v>pal_002</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>捣蛋猫</x:v>
+        <x:v>灰尾狸</x:v>
       </x:c>
       <x:c r="C3" s="3" t="str">
         <x:v>无</x:v>
@@ -745,7 +745,7 @@
       </x:c>
       <x:c r="E3" s="3"/>
       <x:c r="F3" s="3" t="str">
-        <x:v>night_base, elem_无, tier_pT1</x:v>
+        <x:v>night_base, elem_无, tier_pT1, shop_store_37, shop_store_55, shop_store_73</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
         <x:v>24</x:v>
@@ -780,7 +780,7 @@
         <x:v>pal_003</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>皮皮鸡</x:v>
+        <x:v>芦花鸡</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>无</x:v>
@@ -790,7 +790,7 @@
       </x:c>
       <x:c r="E4" s="3"/>
       <x:c r="F4" s="3" t="str">
-        <x:v>night_base, elem_无, tier_pT1</x:v>
+        <x:v>night_base, elem_无, tier_pT1, role_风系铺场, shop_store_37, shop_store_55</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
         <x:v>15</x:v>
@@ -825,7 +825,7 @@
         <x:v>pal_004</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>翠叶鼠</x:v>
+        <x:v>青藤鼠</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>草</x:v>
@@ -835,7 +835,7 @@
       </x:c>
       <x:c r="E5" s="3"/>
       <x:c r="F5" s="3" t="str">
-        <x:v>night_base, elem_草, tier_pT1</x:v>
+        <x:v>night_base, elem_草, tier_pT1, shop_store_37, shop_store_74</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
         <x:v>18</x:v>
@@ -870,7 +870,7 @@
         <x:v>pal_005</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>火绒狐</x:v>
+        <x:v>赤尾狐</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
         <x:v>火</x:v>
@@ -880,7 +880,7 @@
       </x:c>
       <x:c r="E6" s="3"/>
       <x:c r="F6" s="3" t="str">
-        <x:v>night_base, elem_火, tier_pT1</x:v>
+        <x:v>night_base, elem_火, tier_pT1, role_风系铺场, shop_store_56, shop_store_74</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
         <x:v>30</x:v>
@@ -915,7 +915,7 @@
         <x:v>pal_006</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>冲浪鸭</x:v>
+        <x:v>碧水鸭</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>水</x:v>
@@ -925,7 +925,7 @@
       </x:c>
       <x:c r="E7" s="3"/>
       <x:c r="F7" s="3" t="str">
-        <x:v>night_base, elem_水, tier_pT1</x:v>
+        <x:v>night_base, elem_水, tier_pT1, shop_store_38, shop_store_56, shop_store_74</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
         <x:v>18</x:v>
@@ -960,7 +960,7 @@
         <x:v>pal_007</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>伏特喵</x:v>
+        <x:v>雷须猫</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>雷</x:v>
@@ -970,7 +970,7 @@
       </x:c>
       <x:c r="E8" s="3"/>
       <x:c r="F8" s="3" t="str">
-        <x:v>night_base, elem_雷, tier_pT1</x:v>
+        <x:v>night_base, elem_雷, tier_pT1, shop_store_38, shop_store_56, shop_store_74</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
         <x:v>24</x:v>
@@ -1005,7 +1005,7 @@
         <x:v>pal_008</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>新叶猿</x:v>
+        <x:v>藤甲猿</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
         <x:v>草</x:v>
@@ -1017,7 +1017,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F9" s="3" t="str">
-        <x:v>night_base, elem_草, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_草, role_坦克, tier_pT1, role_抗压承伤, shop_store_38, shop_store_56, shop_store_74</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
         <x:v>24</x:v>
@@ -1052,7 +1052,7 @@
         <x:v>pal_009</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>燎火鹿</x:v>
+        <x:v>火角鹿</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
         <x:v>火</x:v>
@@ -1064,7 +1064,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT1, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT1, role_火系压制, shop_store_38, shop_store_56, shop_store_74</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>24</x:v>
@@ -1099,7 +1099,7 @@
         <x:v>pal_010</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>企丸丸</x:v>
+        <x:v>霜羽鹭</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
         <x:v>水、冰</x:v>
@@ -1111,7 +1111,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>night_base, elem_水, elem_冰, role_治疗, tier_pT1, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, elem_冰, role_治疗, tier_pT1, role_水系牵制, shop_store_38, shop_store_56</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
         <x:v>18</x:v>
@@ -1146,7 +1146,7 @@
         <x:v>pal_011</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>企丸王</x:v>
+        <x:v>冰背獭</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
         <x:v>水、冰</x:v>
@@ -1158,7 +1158,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F12" s="3" t="str">
-        <x:v>night_base, elem_水, elem_冰, role_治疗, tier_pT1, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, elem_冰, role_治疗, tier_pT1, role_水系牵制, shop_store_38, shop_store_75</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
         <x:v>24</x:v>
@@ -1205,7 +1205,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F13" s="3" t="str">
-        <x:v>night_base, elem_雷, role_控制, tier_pT1, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, role_控制, tier_pT1, role_风系牵制, shop_store_57, shop_store_75</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
         <x:v>18</x:v>
@@ -1240,7 +1240,7 @@
         <x:v>pal_013</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>叶泥泥</x:v>
+        <x:v>苔甲龟</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
         <x:v>草、地</x:v>
@@ -1252,7 +1252,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F14" s="3" t="str">
-        <x:v>night_base, elem_草, elem_地, role_坦克, tier_pT1, role_重甲抗压</x:v>
+        <x:v>night_base, elem_草, elem_地, role_坦克, tier_pT1, role_重甲抗压, shop_store_39, shop_store_57, shop_store_75</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
         <x:v>20</x:v>
@@ -1287,7 +1287,7 @@
         <x:v>pal_014</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>玉藻狐</x:v>
+        <x:v>金钱狸</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
         <x:v>无</x:v>
@@ -1299,7 +1299,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F15" s="3" t="str">
-        <x:v>night_base, elem_无, role_经济, tier_pT1, role_风系铺场</x:v>
+        <x:v>night_base, elem_无, role_经济, tier_pT1, role_风系铺场, shop_store_39, shop_store_57, shop_store_75</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
         <x:v>15</x:v>
@@ -1334,7 +1334,7 @@
         <x:v>pal_015</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>啼卡尔</x:v>
+        <x:v>黑甲猪</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
         <x:v>暗</x:v>
@@ -1346,7 +1346,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F16" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_重甲抗压</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_重甲抗压, shop_store_39, shop_store_57, shop_store_75</x:v>
       </x:c>
       <x:c r="G16" s="3" t="str">
         <x:v>12</x:v>
@@ -1381,7 +1381,7 @@
         <x:v>pal_016</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>壶小象</x:v>
+        <x:v>涧水象</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
         <x:v>水</x:v>
@@ -1393,7 +1393,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F17" s="3" t="str">
-        <x:v>night_base, elem_水, role_治疗, tier_pT1, role_水系控场</x:v>
+        <x:v>night_base, elem_水, role_治疗, tier_pT1, role_水系控场, shop_store_39, shop_store_57, shop_store_75</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
         <x:v>25</x:v>
@@ -1428,7 +1428,7 @@
         <x:v>pal_017</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>瞅什魔</x:v>
+        <x:v>黑角犀</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
         <x:v>暗</x:v>
@@ -1440,7 +1440,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F18" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_重甲抗压</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_重甲抗压, shop_store_39, shop_store_57</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
         <x:v>40</x:v>
@@ -1475,7 +1475,7 @@
         <x:v>pal_018</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>米露菲</x:v>
+        <x:v>竹囊鼠</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
         <x:v>无</x:v>
@@ -1487,7 +1487,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F19" s="3" t="str">
-        <x:v>night_base, elem_无, role_经济, tier_pT1, role_风系铺场</x:v>
+        <x:v>night_base, elem_无, role_经济, tier_pT1, role_风系铺场, shop_store_39, shop_store_76</x:v>
       </x:c>
       <x:c r="G19" s="3" t="str">
         <x:v>10</x:v>
@@ -1522,7 +1522,7 @@
         <x:v>pal_019</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
-        <x:v>寐魔</x:v>
+        <x:v>夜穴鼹</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
         <x:v>暗</x:v>
@@ -1534,7 +1534,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F20" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_重甲抗压</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_重甲抗压, role_水系控场, shop_store_58, shop_store_76</x:v>
       </x:c>
       <x:c r="G20" s="3" t="str">
         <x:v>30</x:v>
@@ -1569,7 +1569,7 @@
         <x:v>pal_020</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
-        <x:v>草莽猪</x:v>
+        <x:v>沙鬃猪</x:v>
       </x:c>
       <x:c r="C21" s="3" t="str">
         <x:v>地</x:v>
@@ -1581,7 +1581,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F21" s="3" t="str">
-        <x:v>night_base, elem_地, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_地, role_坦克, tier_pT1, role_抗压承伤, role_水系控场, shop_store_40, shop_store_58, shop_store_76</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
         <x:v>15</x:v>
@@ -1616,7 +1616,7 @@
         <x:v>pal_021</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
-        <x:v>露娜蒂</x:v>
+        <x:v>暮羽鸦</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
         <x:v>暗</x:v>
@@ -1628,7 +1628,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F22" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_抗压承伤, role_水系控场, shop_store_40, shop_store_58, shop_store_76</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
         <x:v>15</x:v>
@@ -1663,7 +1663,7 @@
         <x:v>pal_022</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
-        <x:v>遁地鼠</x:v>
+        <x:v>岩爪鼹</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
         <x:v>地</x:v>
@@ -1675,7 +1675,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F23" s="3" t="str">
-        <x:v>night_base, elem_地, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_地, role_坦克, tier_pT1, role_抗压承伤, role_水系控场, shop_store_40, shop_store_58, shop_store_76</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
         <x:v>25</x:v>
@@ -1710,7 +1710,7 @@
         <x:v>pal_023</x:v>
       </x:c>
       <x:c r="B24" s="3" t="str">
-        <x:v>勾魂鱿</x:v>
+        <x:v>墨潭鲵</x:v>
       </x:c>
       <x:c r="C24" s="3" t="str">
         <x:v>暗</x:v>
@@ -1722,7 +1722,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F24" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT1, role_抗压承伤, role_水系控场, shop_store_40, shop_store_58, shop_store_76</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
         <x:v>25</x:v>
@@ -1757,7 +1757,7 @@
         <x:v>pal_024</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
-        <x:v>喵丝特</x:v>
+        <x:v>幽纹猫</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
         <x:v>暗</x:v>
@@ -1769,7 +1769,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F25" s="3" t="str">
-        <x:v>night_base, elem_暗, role_经济, tier_pT1, role_土系抗压</x:v>
+        <x:v>night_base, elem_暗, role_经济, tier_pT1, role_土系抗压, shop_store_40, shop_store_58</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
         <x:v>10</x:v>
@@ -1804,7 +1804,7 @@
         <x:v>pal_025</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>鲁米儿</x:v>
+        <x:v>泉须鲶</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
         <x:v>水</x:v>
@@ -1816,7 +1816,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F26" s="3" t="str">
-        <x:v>night_base, elem_水, role_治疗, tier_pT1, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, role_治疗, tier_pT1, role_水系牵制, shop_store_40, shop_store_77</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
         <x:v>10</x:v>
@@ -1851,7 +1851,7 @@
         <x:v>pal_026</x:v>
       </x:c>
       <x:c r="B27" s="3" t="str">
-        <x:v>猎狼</x:v>
+        <x:v>疾风狼</x:v>
       </x:c>
       <x:c r="C27" s="3" t="str">
         <x:v>无</x:v>
@@ -1863,7 +1863,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F27" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT1, role_抗压承伤, shop_store_59, shop_store_77</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
         <x:v>20</x:v>
@@ -1898,7 +1898,7 @@
         <x:v>pal_027</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>炸蛋鸟</x:v>
+        <x:v>惊羽雀</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
         <x:v>无</x:v>
@@ -1910,7 +1910,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT1, role_机动压制</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT1, role_机动压制, shop_store_41, shop_store_59, shop_store_77</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
         <x:v>20</x:v>
@@ -1945,7 +1945,7 @@
         <x:v>pal_028</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
-        <x:v>波娜兔</x:v>
+        <x:v>药草兔</x:v>
       </x:c>
       <x:c r="C29" s="3" t="str">
         <x:v>草</x:v>
@@ -1957,7 +1957,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F29" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT1, role_风系铺场</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT1, role_风系铺场, shop_store_41, shop_store_59, shop_store_77</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
         <x:v>10</x:v>
@@ -1992,7 +1992,7 @@
         <x:v>pal_029</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>波霸牛</x:v>
+        <x:v>黄背牛</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
         <x:v>无</x:v>
@@ -2004,7 +2004,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F30" s="3" t="str">
-        <x:v>night_base, elem_无, role_经济, tier_pT1, role_诅咒牵制</x:v>
+        <x:v>night_base, elem_无, role_经济, tier_pT1, role_诅咒牵制, role_火系重压, shop_store_41, shop_store_59, shop_store_77</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
         <x:v>25</x:v>
@@ -2039,7 +2039,7 @@
         <x:v>pal_030</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>荆棘魔仙</x:v>
+        <x:v>花刺蛛</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>草</x:v>
@@ -2051,7 +2051,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F31" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT1, role_风系铺场</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT1, role_风系铺场, role_火系重压, shop_store_41, shop_store_59, shop_store_77</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
         <x:v>25</x:v>
@@ -2086,7 +2086,7 @@
         <x:v>pal_031</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
-        <x:v>鲨小子</x:v>
+        <x:v>青背鲵</x:v>
       </x:c>
       <x:c r="C32" s="3" t="str">
         <x:v>水</x:v>
@@ -2098,7 +2098,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F32" s="3" t="str">
-        <x:v>night_base, elem_水, role_治疗, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_水, role_治疗, tier_pT1, role_抗压承伤, role_火系重压, shop_store_41, shop_store_59</x:v>
       </x:c>
       <x:c r="G32" s="3" t="str">
         <x:v>25</x:v>
@@ -2133,7 +2133,7 @@
         <x:v>pal_032</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
-        <x:v>吊缚灵</x:v>
+        <x:v>石甲鲮</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
         <x:v>地</x:v>
@@ -2145,7 +2145,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F33" s="3" t="str">
-        <x:v>night_base, elem_地, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_地, role_坦克, tier_pT1, role_抗压承伤, role_火系重压, shop_store_41, shop_store_78</x:v>
       </x:c>
       <x:c r="G33" s="3" t="str">
         <x:v>30</x:v>
@@ -2180,7 +2180,7 @@
         <x:v>pal_033</x:v>
       </x:c>
       <x:c r="B34" s="3" t="str">
-        <x:v>叶胖达</x:v>
+        <x:v>芭蕉熊</x:v>
       </x:c>
       <x:c r="C34" s="3" t="str">
         <x:v>草</x:v>
@@ -2192,7 +2192,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F34" s="3" t="str">
-        <x:v>night_base, elem_草, role_坦克, tier_pT1, role_抗压承伤</x:v>
+        <x:v>night_base, elem_草, role_坦克, tier_pT1, role_抗压承伤, shop_store_60, shop_store_78</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
         <x:v>15</x:v>
@@ -2227,7 +2227,7 @@
         <x:v>pal_034</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
-        <x:v>棉花糖</x:v>
+        <x:v>蜜纹獾</x:v>
       </x:c>
       <x:c r="C35" s="3" t="str">
         <x:v>无</x:v>
@@ -2239,7 +2239,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F35" s="3" t="str">
-        <x:v>night_base, elem_无, role_经济, tier_pT1, role_远点压制</x:v>
+        <x:v>night_base, elem_无, role_经济, tier_pT1, role_远点压制, shop_store_42, shop_store_60, shop_store_78</x:v>
       </x:c>
       <x:c r="G35" s="3" t="str">
         <x:v>10</x:v>
@@ -2274,7 +2274,7 @@
         <x:v>pal_035</x:v>
       </x:c>
       <x:c r="B36" s="3" t="str">
-        <x:v>灌木羊</x:v>
+        <x:v>藤巢蜂</x:v>
       </x:c>
       <x:c r="C36" s="3" t="str">
         <x:v>草</x:v>
@@ -2286,7 +2286,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F36" s="3" t="str">
-        <x:v>night_base, elem_草, role_召唤, tier_pT1, role_召唤铺场</x:v>
+        <x:v>night_base, elem_草, role_召唤, tier_pT1, role_召唤铺场, shop_store_42, shop_store_60, shop_store_78</x:v>
       </x:c>
       <x:c r="G36" s="3" t="str">
         <x:v>10</x:v>
@@ -2321,7 +2321,7 @@
         <x:v>pal_036</x:v>
       </x:c>
       <x:c r="B37" s="3" t="str">
-        <x:v>美露帕</x:v>
+        <x:v>云纹巨驼</x:v>
       </x:c>
       <x:c r="C37" s="3" t="str">
         <x:v>无</x:v>
@@ -2333,7 +2333,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F37" s="3" t="str">
-        <x:v>night_base, elem_无, role_经济, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_无, role_经济, tier_pT2, role_远点压制, shop_store_42, shop_store_60, shop_store_78</x:v>
       </x:c>
       <x:c r="G37" s="3" t="str">
         <x:v>20</x:v>
@@ -2368,7 +2368,7 @@
         <x:v>pal_037</x:v>
       </x:c>
       <x:c r="B38" s="3" t="str">
-        <x:v>紫霞鹿</x:v>
+        <x:v>月角白鹿</x:v>
       </x:c>
       <x:c r="C38" s="3" t="str">
         <x:v>无</x:v>
@@ -2380,7 +2380,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F38" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制, shop_store_42, shop_store_60, shop_store_78</x:v>
       </x:c>
       <x:c r="G38" s="3" t="str">
         <x:v>10</x:v>
@@ -2415,7 +2415,7 @@
         <x:v>pal_038</x:v>
       </x:c>
       <x:c r="B39" s="3" t="str">
-        <x:v>疾风隼</x:v>
+        <x:v>疾风苍鹰</x:v>
       </x:c>
       <x:c r="C39" s="3" t="str">
         <x:v>无</x:v>
@@ -2427,7 +2427,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F39" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制, shop_store_42, shop_store_60</x:v>
       </x:c>
       <x:c r="G39" s="3" t="str">
         <x:v>10</x:v>
@@ -2462,7 +2462,7 @@
         <x:v>pal_039</x:v>
       </x:c>
       <x:c r="B40" s="3" t="str">
-        <x:v>姬小兔</x:v>
+        <x:v>银背巨兔</x:v>
       </x:c>
       <x:c r="C40" s="3" t="str">
         <x:v>无</x:v>
@@ -2474,7 +2474,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F40" s="3" t="str">
-        <x:v>night_base, elem_无, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_无, role_坦克, tier_pT2, role_抗压承伤, shop_store_42</x:v>
       </x:c>
       <x:c r="G40" s="3" t="str">
         <x:v>15</x:v>
@@ -2509,7 +2509,7 @@
         <x:v>pal_040</x:v>
       </x:c>
       <x:c r="B41" s="3" t="str">
-        <x:v>炎魔羊</x:v>
+        <x:v>炎角黑羊</x:v>
       </x:c>
       <x:c r="C41" s="3" t="str">
         <x:v>火、暗</x:v>
@@ -2521,7 +2521,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F41" s="3" t="str">
-        <x:v>night_base, elem_火, elem_暗, role_输出, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, elem_暗, role_输出, tier_pT2, role_火系压制, shop_store_61</x:v>
       </x:c>
       <x:c r="G41" s="3" t="str">
         <x:v>25</x:v>
@@ -2556,7 +2556,7 @@
         <x:v>pal_041</x:v>
       </x:c>
       <x:c r="B42" s="3" t="str">
-        <x:v>幻悦蝶</x:v>
+        <x:v>回春彩蝶</x:v>
       </x:c>
       <x:c r="C42" s="3" t="str">
         <x:v>草</x:v>
@@ -2568,7 +2568,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F42" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制, shop_store_43, shop_store_61</x:v>
       </x:c>
       <x:c r="G42" s="3" t="str">
         <x:v>25</x:v>
@@ -2603,7 +2603,7 @@
         <x:v>pal_042</x:v>
       </x:c>
       <x:c r="B43" s="3" t="str">
-        <x:v>炽焰牛</x:v>
+        <x:v>赤焰蛮牛</x:v>
       </x:c>
       <x:c r="C43" s="3" t="str">
         <x:v>火</x:v>
@@ -2615,7 +2615,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F43" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制, shop_store_43, shop_store_61</x:v>
       </x:c>
       <x:c r="G43" s="3" t="str">
         <x:v>10</x:v>
@@ -2650,7 +2650,7 @@
         <x:v>pal_043</x:v>
       </x:c>
       <x:c r="B44" s="3" t="str">
-        <x:v>趴趴鲶</x:v>
+        <x:v>泥甲巨鲶</x:v>
       </x:c>
       <x:c r="C44" s="3" t="str">
         <x:v>地</x:v>
@@ -2662,7 +2662,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F44" s="3" t="str">
-        <x:v>night_base, elem_地, role_治疗, tier_pT2, role_土系抗压</x:v>
+        <x:v>night_base, elem_地, role_治疗, tier_pT2, role_土系抗压, shop_store_43, shop_store_61</x:v>
       </x:c>
       <x:c r="G44" s="3" t="str">
         <x:v>25</x:v>
@@ -2697,7 +2697,7 @@
         <x:v>pal_044</x:v>
       </x:c>
       <x:c r="B45" s="3" t="str">
-        <x:v>黑鸦隐士</x:v>
+        <x:v>夜羽巨鸦</x:v>
       </x:c>
       <x:c r="C45" s="3" t="str">
         <x:v>暗</x:v>
@@ -2709,7 +2709,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F45" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤, role_夹击牵制, shop_store_43, shop_store_61</x:v>
       </x:c>
       <x:c r="G45" s="3" t="str">
         <x:v>15</x:v>
@@ -2744,7 +2744,7 @@
         <x:v>pal_045</x:v>
       </x:c>
       <x:c r="B46" s="3" t="str">
-        <x:v>朋克蜥</x:v>
+        <x:v>墨鳞巨蜥</x:v>
       </x:c>
       <x:c r="C46" s="3" t="str">
         <x:v>暗</x:v>
@@ -2756,7 +2756,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F46" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤, role_夹击牵制, shop_store_43, shop_store_61</x:v>
       </x:c>
       <x:c r="G46" s="3" t="str">
         <x:v>15</x:v>
@@ -2791,7 +2791,7 @@
         <x:v>pal_046</x:v>
       </x:c>
       <x:c r="B47" s="3" t="str">
-        <x:v>月镰魔</x:v>
+        <x:v>月镰螳螂</x:v>
       </x:c>
       <x:c r="C47" s="3" t="str">
         <x:v>暗</x:v>
@@ -2803,7 +2803,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F47" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤, role_夹击牵制, shop_store_43</x:v>
       </x:c>
       <x:c r="G47" s="3" t="str">
         <x:v>30</x:v>
@@ -2838,7 +2838,7 @@
         <x:v>pal_047</x:v>
       </x:c>
       <x:c r="B48" s="3" t="str">
-        <x:v>天擒鸟</x:v>
+        <x:v>裂空苍鹰</x:v>
       </x:c>
       <x:c r="C48" s="3" t="str">
         <x:v>无</x:v>
@@ -2850,7 +2850,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F48" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制, shop_store_62</x:v>
       </x:c>
       <x:c r="G48" s="3" t="str">
         <x:v>10</x:v>
@@ -2885,7 +2885,7 @@
         <x:v>pal_048</x:v>
       </x:c>
       <x:c r="B49" s="3" t="str">
-        <x:v>羽箭射手</x:v>
+        <x:v>木刺豪猪</x:v>
       </x:c>
       <x:c r="C49" s="3" t="str">
         <x:v>草</x:v>
@@ -2897,7 +2897,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F49" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制, role_夹击牵制, shop_store_44, shop_store_62</x:v>
       </x:c>
       <x:c r="G49" s="3" t="str">
         <x:v>25</x:v>
@@ -2932,7 +2932,7 @@
         <x:v>pal_049</x:v>
       </x:c>
       <x:c r="B50" s="3" t="str">
-        <x:v>铁拳猿</x:v>
+        <x:v>铁臂黑猿</x:v>
       </x:c>
       <x:c r="C50" s="3" t="str">
         <x:v>无</x:v>
@@ -2944,7 +2944,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F50" s="3" t="str">
-        <x:v>night_base, elem_无, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_无, role_坦克, tier_pT2, role_抗压承伤, role_夹击牵制, shop_store_44, shop_store_62</x:v>
       </x:c>
       <x:c r="G50" s="3" t="str">
         <x:v>15</x:v>
@@ -2979,7 +2979,7 @@
         <x:v>pal_050</x:v>
       </x:c>
       <x:c r="B51" s="3" t="str">
-        <x:v>骑士蜂</x:v>
+        <x:v>金甲蜂群</x:v>
       </x:c>
       <x:c r="C51" s="3" t="str">
         <x:v>草</x:v>
@@ -2991,7 +2991,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F51" s="3" t="str">
-        <x:v>night_base, elem_草, role_召唤, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_草, role_召唤, tier_pT2, role_召唤铺场, shop_store_44, shop_store_62</x:v>
       </x:c>
       <x:c r="G51" s="3" t="str">
         <x:v>35</x:v>
@@ -3026,7 +3026,7 @@
         <x:v>pal_051</x:v>
       </x:c>
       <x:c r="B52" s="3" t="str">
-        <x:v>女皇蜂</x:v>
+        <x:v>百花巨蜂</x:v>
       </x:c>
       <x:c r="C52" s="3" t="str">
         <x:v>草</x:v>
@@ -3038,7 +3038,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F52" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制, shop_store_44, shop_store_62</x:v>
       </x:c>
       <x:c r="G52" s="3" t="str">
         <x:v>25</x:v>
@@ -3073,7 +3073,7 @@
         <x:v>pal_052</x:v>
       </x:c>
       <x:c r="B53" s="3" t="str">
-        <x:v>笑魇猫</x:v>
+        <x:v>笑面山猫</x:v>
       </x:c>
       <x:c r="C53" s="3" t="str">
         <x:v>无</x:v>
@@ -3085,7 +3085,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F53" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制, shop_store_44, shop_store_62</x:v>
       </x:c>
       <x:c r="G53" s="3" t="str">
         <x:v>10</x:v>
@@ -3120,7 +3120,7 @@
         <x:v>pal_053</x:v>
       </x:c>
       <x:c r="B54" s="3" t="str">
-        <x:v>毛掸儿</x:v>
+        <x:v>霜尾雪貂</x:v>
       </x:c>
       <x:c r="C54" s="3" t="str">
         <x:v>冰</x:v>
@@ -3132,7 +3132,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F54" s="3" t="str">
-        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制, shop_store_44</x:v>
       </x:c>
       <x:c r="G54" s="3" t="str">
         <x:v>20</x:v>
@@ -3167,7 +3167,7 @@
         <x:v>pal_054</x:v>
       </x:c>
       <x:c r="B55" s="3" t="str">
-        <x:v>毛老爹</x:v>
+        <x:v>白眉雪猿</x:v>
       </x:c>
       <x:c r="C55" s="3" t="str">
         <x:v>冰</x:v>
@@ -3179,7 +3179,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F55" s="3" t="str">
-        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制, shop_store_63</x:v>
       </x:c>
       <x:c r="G55" s="3" t="str">
         <x:v>20</x:v>
@@ -3214,7 +3214,7 @@
         <x:v>pal_055</x:v>
       </x:c>
       <x:c r="B56" s="3" t="str">
-        <x:v>疾旋鼬</x:v>
+        <x:v>寒风幼螭</x:v>
       </x:c>
       <x:c r="C56" s="3" t="str">
         <x:v>冰、龙</x:v>
@@ -3226,7 +3226,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F56" s="3" t="str">
-        <x:v>night_base, elem_冰, elem_龙, role_控制, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_冰, elem_龙, role_控制, tier_pT2, role_召唤铺场, shop_store_45, shop_store_63</x:v>
       </x:c>
       <x:c r="G56" s="3" t="str">
         <x:v>30</x:v>
@@ -3261,7 +3261,7 @@
         <x:v>pal_056</x:v>
       </x:c>
       <x:c r="B57" s="3" t="str">
-        <x:v>雷角马</x:v>
+        <x:v>震角雷牛</x:v>
       </x:c>
       <x:c r="C57" s="3" t="str">
         <x:v>雷</x:v>
@@ -3273,7 +3273,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F57" s="3" t="str">
-        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制, shop_store_45, shop_store_63</x:v>
       </x:c>
       <x:c r="G57" s="3" t="str">
         <x:v>20</x:v>
@@ -3308,7 +3308,7 @@
         <x:v>pal_057</x:v>
       </x:c>
       <x:c r="B58" s="3" t="str">
-        <x:v>吹雪狐</x:v>
+        <x:v>吹雪银狐</x:v>
       </x:c>
       <x:c r="C58" s="3" t="str">
         <x:v>冰</x:v>
@@ -3320,7 +3320,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F58" s="3" t="str">
-        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制, shop_store_45, shop_store_63</x:v>
       </x:c>
       <x:c r="G58" s="3" t="str">
         <x:v>20</x:v>
@@ -3355,7 +3355,7 @@
         <x:v>pal_058</x:v>
       </x:c>
       <x:c r="B59" s="3" t="str">
-        <x:v>火麒麟</x:v>
+        <x:v>丹角火麟</x:v>
       </x:c>
       <x:c r="C59" s="3" t="str">
         <x:v>火</x:v>
@@ -3367,7 +3367,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F59" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制, shop_store_45, shop_store_63</x:v>
       </x:c>
       <x:c r="G59" s="3" t="str">
         <x:v>30</x:v>
@@ -3402,7 +3402,7 @@
         <x:v>pal_059</x:v>
       </x:c>
       <x:c r="B60" s="3" t="str">
-        <x:v>严冬鹿</x:v>
+        <x:v>冰角白鹿</x:v>
       </x:c>
       <x:c r="C60" s="3" t="str">
         <x:v>冰</x:v>
@@ -3414,7 +3414,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F60" s="3" t="str">
-        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, role_控制, tier_pT2, role_水系牵制, shop_store_45, shop_store_63</x:v>
       </x:c>
       <x:c r="G60" s="3" t="str">
         <x:v>20</x:v>
@@ -3449,7 +3449,7 @@
         <x:v>pal_060</x:v>
       </x:c>
       <x:c r="B61" s="3" t="str">
-        <x:v>霹雳犬</x:v>
+        <x:v>霹雳战獒</x:v>
       </x:c>
       <x:c r="C61" s="3" t="str">
         <x:v>雷</x:v>
@@ -3461,7 +3461,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F61" s="3" t="str">
-        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制, shop_store_45</x:v>
       </x:c>
       <x:c r="G61" s="3" t="str">
         <x:v>20</x:v>
@@ -3496,7 +3496,7 @@
         <x:v>pal_061</x:v>
       </x:c>
       <x:c r="B62" s="3" t="str">
-        <x:v>苍焰狼</x:v>
+        <x:v>苍焰赤豺</x:v>
       </x:c>
       <x:c r="C62" s="3" t="str">
         <x:v>火</x:v>
@@ -3508,7 +3508,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F62" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_成长输出</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_成长输出, shop_store_64</x:v>
       </x:c>
       <x:c r="G62" s="3" t="str">
         <x:v>25</x:v>
@@ -3543,7 +3543,7 @@
         <x:v>pal_062</x:v>
       </x:c>
       <x:c r="B63" s="3" t="str">
-        <x:v>雷鸣童子</x:v>
+        <x:v>雷纹巨猿</x:v>
       </x:c>
       <x:c r="C63" s="3" t="str">
         <x:v>雷</x:v>
@@ -3555,7 +3555,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F63" s="3" t="str">
-        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制, shop_store_46, shop_store_64</x:v>
       </x:c>
       <x:c r="G63" s="3" t="str">
         <x:v>20</x:v>
@@ -3590,7 +3590,7 @@
         <x:v>pal_063</x:v>
       </x:c>
       <x:c r="B64" s="3" t="str">
-        <x:v>秘斯媞雅</x:v>
+        <x:v>蜃雾白鹿</x:v>
       </x:c>
       <x:c r="C64" s="3" t="str">
         <x:v>无</x:v>
@@ -3602,7 +3602,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F64" s="3" t="str">
-        <x:v>night_base, elem_无, role_召唤, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_无, role_召唤, tier_pT2, role_召唤铺场, shop_store_46, shop_store_64</x:v>
       </x:c>
       <x:c r="G64" s="3" t="str">
         <x:v>20</x:v>
@@ -3637,7 +3637,7 @@
         <x:v>pal_064</x:v>
       </x:c>
       <x:c r="B65" s="3" t="str">
-        <x:v>花冠龙</x:v>
+        <x:v>翠冠花螭</x:v>
       </x:c>
       <x:c r="C65" s="3" t="str">
         <x:v>草、龙</x:v>
@@ -3649,7 +3649,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F65" s="3" t="str">
-        <x:v>night_base, elem_草, elem_龙, role_召唤, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_草, elem_龙, role_召唤, tier_pT2, role_召唤铺场, shop_store_46, shop_store_64</x:v>
       </x:c>
       <x:c r="G65" s="3" t="str">
         <x:v>35</x:v>
@@ -3684,7 +3684,7 @@
         <x:v>pal_065</x:v>
       </x:c>
       <x:c r="B66" s="3" t="str">
-        <x:v>雷冠龙</x:v>
+        <x:v>霆角龙犀</x:v>
       </x:c>
       <x:c r="C66" s="3" t="str">
         <x:v>雷、龙</x:v>
@@ -3696,7 +3696,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F66" s="3" t="str">
-        <x:v>night_base, elem_雷, elem_龙, role_控制, tier_pT2, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, elem_龙, role_控制, tier_pT2, role_风系牵制, shop_store_46, shop_store_64</x:v>
       </x:c>
       <x:c r="G66" s="3" t="str">
         <x:v>35</x:v>
@@ -3731,7 +3731,7 @@
         <x:v>pal_066</x:v>
       </x:c>
       <x:c r="B67" s="3" t="str">
-        <x:v>滑水蛇</x:v>
+        <x:v>浪鳞水蛇</x:v>
       </x:c>
       <x:c r="C67" s="3" t="str">
         <x:v>水</x:v>
@@ -3743,7 +3743,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F67" s="3" t="str">
-        <x:v>night_base, elem_水, role_治疗, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, role_治疗, tier_pT2, role_水系牵制, shop_store_46, shop_store_64</x:v>
       </x:c>
       <x:c r="G67" s="3" t="str">
         <x:v>25</x:v>
@@ -3778,7 +3778,7 @@
         <x:v>pal_067</x:v>
       </x:c>
       <x:c r="B68" s="3" t="str">
-        <x:v>流沙蛇</x:v>
+        <x:v>沙鳞巨蟒</x:v>
       </x:c>
       <x:c r="C68" s="3" t="str">
         <x:v>地</x:v>
@@ -3790,7 +3790,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F68" s="3" t="str">
-        <x:v>night_base, elem_地, role_坦克, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_地, role_坦克, tier_pT2, role_召唤铺场, shop_store_46</x:v>
       </x:c>
       <x:c r="G68" s="3" t="str">
         <x:v>20</x:v>
@@ -3825,7 +3825,7 @@
         <x:v>pal_068</x:v>
       </x:c>
       <x:c r="B69" s="3" t="str">
-        <x:v>噬魂兽</x:v>
+        <x:v>食梦黑貘</x:v>
       </x:c>
       <x:c r="C69" s="3" t="str">
         <x:v>暗</x:v>
@@ -3837,7 +3837,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F69" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤, shop_store_65</x:v>
       </x:c>
       <x:c r="G69" s="3" t="str">
         <x:v>25</x:v>
@@ -3872,7 +3872,7 @@
         <x:v>pal_069</x:v>
       </x:c>
       <x:c r="B70" s="3" t="str">
-        <x:v>碎岩龟</x:v>
+        <x:v>碎岩巨龟</x:v>
       </x:c>
       <x:c r="C70" s="3" t="str">
         <x:v>地</x:v>
@@ -3884,7 +3884,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F70" s="3" t="str">
-        <x:v>night_base, elem_地, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_地, role_坦克, tier_pT2, role_抗压承伤, shop_store_47, shop_store_65</x:v>
       </x:c>
       <x:c r="G70" s="3" t="str">
         <x:v>25</x:v>
@@ -3919,7 +3919,7 @@
         <x:v>pal_070</x:v>
       </x:c>
       <x:c r="B71" s="3" t="str">
-        <x:v>猫蝠怪</x:v>
+        <x:v>猫翼夜蝠</x:v>
       </x:c>
       <x:c r="C71" s="3" t="str">
         <x:v>暗</x:v>
@@ -3931,7 +3931,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F71" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_抗压承伤, shop_store_47, shop_store_65</x:v>
       </x:c>
       <x:c r="G71" s="3" t="str">
         <x:v>25</x:v>
@@ -3966,7 +3966,7 @@
         <x:v>pal_071</x:v>
       </x:c>
       <x:c r="B72" s="3" t="str">
-        <x:v>博爱蜥</x:v>
+        <x:v>甘露壁虎</x:v>
       </x:c>
       <x:c r="C72" s="3" t="str">
         <x:v>无</x:v>
@@ -3978,7 +3978,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F72" s="3" t="str">
-        <x:v>night_base, elem_无, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_无, role_治疗, tier_pT2, role_远点压制, shop_store_47, shop_store_65</x:v>
       </x:c>
       <x:c r="G72" s="3" t="str">
         <x:v>25</x:v>
@@ -4013,7 +4013,7 @@
         <x:v>pal_072</x:v>
       </x:c>
       <x:c r="B73" s="3" t="str">
-        <x:v>融焰娘</x:v>
+        <x:v>赤巢火蚁</x:v>
       </x:c>
       <x:c r="C73" s="3" t="str">
         <x:v>火</x:v>
@@ -4025,7 +4025,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F73" s="3" t="str">
-        <x:v>night_base, elem_火, role_召唤, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_火, role_召唤, tier_pT2, role_召唤铺场, shop_store_47, shop_store_65</x:v>
       </x:c>
       <x:c r="G73" s="3" t="str">
         <x:v>20</x:v>
@@ -4060,7 +4060,7 @@
         <x:v>pal_073</x:v>
       </x:c>
       <x:c r="B74" s="3" t="str">
-        <x:v>烽歌龙</x:v>
+        <x:v>烽翼火龙</x:v>
       </x:c>
       <x:c r="C74" s="3" t="str">
         <x:v>火、暗</x:v>
@@ -4072,7 +4072,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F74" s="3" t="str">
-        <x:v>night_base, elem_火, elem_暗, role_机动, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, elem_暗, role_机动, tier_pT2, role_火系压制, role_成长输出, shop_store_47, shop_store_65</x:v>
       </x:c>
       <x:c r="G74" s="3" t="str">
         <x:v>30</x:v>
@@ -4107,7 +4107,7 @@
         <x:v>pal_074</x:v>
       </x:c>
       <x:c r="B75" s="3" t="str">
-        <x:v>霜歌龙</x:v>
+        <x:v>霜翼冥龙</x:v>
       </x:c>
       <x:c r="C75" s="3" t="str">
         <x:v>冰、暗</x:v>
@@ -4119,7 +4119,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F75" s="3" t="str">
-        <x:v>night_base, elem_冰, elem_暗, role_控制, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, elem_暗, role_控制, tier_pT2, role_水系牵制, role_成长输出, shop_store_47</x:v>
       </x:c>
       <x:c r="G75" s="3" t="str">
         <x:v>35</x:v>
@@ -4154,7 +4154,7 @@
         <x:v>pal_075</x:v>
       </x:c>
       <x:c r="B76" s="3" t="str">
-        <x:v>浪刃武士</x:v>
+        <x:v>赤刃螳螂</x:v>
       </x:c>
       <x:c r="C76" s="3" t="str">
         <x:v>火</x:v>
@@ -4166,7 +4166,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F76" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制, shop_store_66</x:v>
       </x:c>
       <x:c r="G76" s="3" t="str">
         <x:v>30</x:v>
@@ -4201,7 +4201,7 @@
         <x:v>pal_076</x:v>
       </x:c>
       <x:c r="B77" s="3" t="str">
-        <x:v>迅雷鸟</x:v>
+        <x:v>迅雷金雕</x:v>
       </x:c>
       <x:c r="C77" s="3" t="str">
         <x:v>雷</x:v>
@@ -4213,7 +4213,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F77" s="3" t="str">
-        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, role_控制, tier_pT2, role_风系牵制, role_成长输出, shop_store_48, shop_store_66</x:v>
       </x:c>
       <x:c r="G77" s="3" t="str">
         <x:v>70</x:v>
@@ -4248,7 +4248,7 @@
         <x:v>pal_077</x:v>
       </x:c>
       <x:c r="B78" s="3" t="str">
-        <x:v>燧火鸟</x:v>
+        <x:v>燧火黑乌</x:v>
       </x:c>
       <x:c r="C78" s="3" t="str">
         <x:v>火</x:v>
@@ -4260,7 +4260,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F78" s="3" t="str">
-        <x:v>night_base, elem_火, role_机动, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_机动, tier_pT2, role_火系压制, role_成长输出, shop_store_48, shop_store_66</x:v>
       </x:c>
       <x:c r="G78" s="3" t="str">
         <x:v>35</x:v>
@@ -4295,7 +4295,7 @@
         <x:v>pal_078</x:v>
       </x:c>
       <x:c r="B79" s="3" t="str">
-        <x:v>暗巫猫</x:v>
+        <x:v>幽泉灵猫</x:v>
       </x:c>
       <x:c r="C79" s="3" t="str">
         <x:v>暗</x:v>
@@ -4307,7 +4307,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F79" s="3" t="str">
-        <x:v>night_base, elem_暗, role_治疗, tier_pT2, role_土系抗压</x:v>
+        <x:v>night_base, elem_暗, role_治疗, tier_pT2, role_土系抗压, shop_store_48, shop_store_66</x:v>
       </x:c>
       <x:c r="G79" s="3" t="str">
         <x:v>25</x:v>
@@ -4342,7 +4342,7 @@
         <x:v>pal_079</x:v>
       </x:c>
       <x:c r="B80" s="3" t="str">
-        <x:v>焰巫狐</x:v>
+        <x:v>焰尾山狐</x:v>
       </x:c>
       <x:c r="C80" s="3" t="str">
         <x:v>火</x:v>
@@ -4354,7 +4354,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F80" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_成长输出</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_成长输出, shop_store_48, shop_store_66</x:v>
       </x:c>
       <x:c r="G80" s="3" t="str">
         <x:v>35</x:v>
@@ -4389,7 +4389,7 @@
         <x:v>pal_080</x:v>
       </x:c>
       <x:c r="B81" s="3" t="str">
-        <x:v>踏春兔</x:v>
+        <x:v>踏春白兔</x:v>
       </x:c>
       <x:c r="C81" s="3" t="str">
         <x:v>草</x:v>
@@ -4401,7 +4401,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F81" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制, shop_store_48, shop_store_66</x:v>
       </x:c>
       <x:c r="G81" s="3" t="str">
         <x:v>25</x:v>
@@ -4436,7 +4436,7 @@
         <x:v>pal_081</x:v>
       </x:c>
       <x:c r="B82" s="3" t="str">
-        <x:v>薇莉塔</x:v>
+        <x:v>药香花鹿</x:v>
       </x:c>
       <x:c r="C82" s="3" t="str">
         <x:v>草</x:v>
@@ -4448,7 +4448,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F82" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制, shop_store_48</x:v>
       </x:c>
       <x:c r="G82" s="3" t="str">
         <x:v>25</x:v>
@@ -4483,7 +4483,7 @@
         <x:v>pal_082</x:v>
       </x:c>
       <x:c r="B83" s="3" t="str">
-        <x:v>绸笠蛾</x:v>
+        <x:v>冰丝巨蛾</x:v>
       </x:c>
       <x:c r="C83" s="3" t="str">
         <x:v>冰</x:v>
@@ -4495,7 +4495,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F83" s="3" t="str">
-        <x:v>night_base, elem_冰, role_治疗, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, role_治疗, tier_pT2, role_水系牵制, role_诅咒牵制, shop_store_67</x:v>
       </x:c>
       <x:c r="G83" s="3" t="str">
         <x:v>25</x:v>
@@ -4530,7 +4530,7 @@
         <x:v>pal_083</x:v>
       </x:c>
       <x:c r="B84" s="3" t="str">
-        <x:v>精灵龙</x:v>
+        <x:v>云鳞幼螭</x:v>
       </x:c>
       <x:c r="C84" s="3" t="str">
         <x:v>龙</x:v>
@@ -4542,7 +4542,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F84" s="3" t="str">
-        <x:v>night_base, elem_龙, role_召唤, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_龙, role_召唤, tier_pT2, role_召唤铺场, role_诅咒牵制, shop_store_49, shop_store_67</x:v>
       </x:c>
       <x:c r="G84" s="3" t="str">
         <x:v>35</x:v>
@@ -4577,7 +4577,7 @@
         <x:v>pal_084</x:v>
       </x:c>
       <x:c r="B85" s="3" t="str">
-        <x:v>水灵龙</x:v>
+        <x:v>沧浪青蛟</x:v>
       </x:c>
       <x:c r="C85" s="3" t="str">
         <x:v>龙、水</x:v>
@@ -4589,7 +4589,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F85" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_水, role_治疗, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_龙, elem_水, role_治疗, tier_pT2, role_水系牵制, role_诅咒牵制, shop_store_49, shop_store_67</x:v>
       </x:c>
       <x:c r="G85" s="3" t="str">
         <x:v>40</x:v>
@@ -4624,7 +4624,7 @@
         <x:v>pal_085</x:v>
       </x:c>
       <x:c r="B86" s="3" t="str">
-        <x:v>水灵儿</x:v>
+        <x:v>涌泉水獭</x:v>
       </x:c>
       <x:c r="C86" s="3" t="str">
         <x:v>水</x:v>
@@ -4636,7 +4636,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F86" s="3" t="str">
-        <x:v>night_base, elem_水, role_治疗, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, role_治疗, tier_pT2, role_水系牵制, role_诅咒牵制, shop_store_49, shop_store_67</x:v>
       </x:c>
       <x:c r="G86" s="3" t="str">
         <x:v>25</x:v>
@@ -4671,7 +4671,7 @@
         <x:v>pal_086</x:v>
       </x:c>
       <x:c r="B87" s="3" t="str">
-        <x:v>火灵儿</x:v>
+        <x:v>赤炎狻猊</x:v>
       </x:c>
       <x:c r="C87" s="3" t="str">
         <x:v>火</x:v>
@@ -4683,7 +4683,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F87" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系压制, shop_store_49, shop_store_67</x:v>
       </x:c>
       <x:c r="G87" s="3" t="str">
         <x:v>30</x:v>
@@ -4718,7 +4718,7 @@
         <x:v>pal_087</x:v>
       </x:c>
       <x:c r="B88" s="3" t="str">
-        <x:v>碧海龙</x:v>
+        <x:v>碧海青蛟</x:v>
       </x:c>
       <x:c r="C88" s="3" t="str">
         <x:v>水、龙</x:v>
@@ -4730,7 +4730,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F88" s="3" t="str">
-        <x:v>night_base, elem_水, elem_龙, role_治疗, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, elem_龙, role_治疗, tier_pT2, role_水系牵制, shop_store_49, shop_store_67</x:v>
       </x:c>
       <x:c r="G88" s="3" t="str">
         <x:v>40</x:v>
@@ -4765,7 +4765,7 @@
         <x:v>pal_088</x:v>
       </x:c>
       <x:c r="B89" s="3" t="str">
-        <x:v>冰棘兽</x:v>
+        <x:v>冰棘豪猪</x:v>
       </x:c>
       <x:c r="C89" s="3" t="str">
         <x:v>冰</x:v>
@@ -4777,7 +4777,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F89" s="3" t="str">
-        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_抗压承伤, shop_store_49</x:v>
       </x:c>
       <x:c r="G89" s="3" t="str">
         <x:v>15</x:v>
@@ -4812,7 +4812,7 @@
         <x:v>pal_089</x:v>
       </x:c>
       <x:c r="B90" s="3" t="str">
-        <x:v>狱焰王</x:v>
+        <x:v>狱火凶獒</x:v>
       </x:c>
       <x:c r="C90" s="3" t="str">
         <x:v>火</x:v>
@@ -4824,7 +4824,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F90" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_重甲抗压</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_重甲抗压, shop_store_68</x:v>
       </x:c>
       <x:c r="G90" s="3" t="str">
         <x:v>40</x:v>
@@ -4859,7 +4859,7 @@
         <x:v>pal_090</x:v>
       </x:c>
       <x:c r="B91" s="3" t="str">
-        <x:v>狱阎王</x:v>
+        <x:v>三首火犬</x:v>
       </x:c>
       <x:c r="C91" s="3" t="str">
         <x:v>火、暗</x:v>
@@ -4871,7 +4871,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F91" s="3" t="str">
-        <x:v>night_base, elem_火, elem_暗, role_输出, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_火, elem_暗, role_输出, tier_pT2, role_召唤铺场, shop_store_50, shop_store_68</x:v>
       </x:c>
       <x:c r="G91" s="3" t="str">
         <x:v>70</x:v>
@@ -4906,7 +4906,7 @@
         <x:v>pal_091</x:v>
       </x:c>
       <x:c r="B92" s="3" t="str">
-        <x:v>佩克龙</x:v>
+        <x:v>覆水龙龟</x:v>
       </x:c>
       <x:c r="C92" s="3" t="str">
         <x:v>龙、水</x:v>
@@ -4918,7 +4918,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F92" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_水, role_坦克, tier_pT2, role_重甲抗压</x:v>
+        <x:v>night_base, elem_龙, elem_水, role_坦克, tier_pT2, role_重甲抗压, shop_store_50, shop_store_68</x:v>
       </x:c>
       <x:c r="G92" s="3" t="str">
         <x:v>35</x:v>
@@ -4953,7 +4953,7 @@
         <x:v>pal_092</x:v>
       </x:c>
       <x:c r="B93" s="3" t="str">
-        <x:v>派克龙</x:v>
+        <x:v>雷泽青蛟</x:v>
       </x:c>
       <x:c r="C93" s="3" t="str">
         <x:v>龙、雷</x:v>
@@ -4965,7 +4965,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F93" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_雷, role_控制, tier_pT2, role_风系牵制</x:v>
+        <x:v>night_base, elem_龙, elem_雷, role_控制, tier_pT2, role_风系牵制, shop_store_50, shop_store_68</x:v>
       </x:c>
       <x:c r="G93" s="3" t="str">
         <x:v>35</x:v>
@@ -5000,7 +5000,7 @@
         <x:v>pal_093</x:v>
       </x:c>
       <x:c r="B94" s="3" t="str">
-        <x:v>连理龙</x:v>
+        <x:v>连理双鹿</x:v>
       </x:c>
       <x:c r="C94" s="3" t="str">
         <x:v>草</x:v>
@@ -5012,7 +5012,7 @@
         <x:v>召唤</x:v>
       </x:c>
       <x:c r="F94" s="3" t="str">
-        <x:v>night_base, elem_草, role_召唤, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_草, role_召唤, tier_pT2, role_召唤铺场, shop_store_50, shop_store_68</x:v>
       </x:c>
       <x:c r="G94" s="3" t="str">
         <x:v>35</x:v>
@@ -5047,7 +5047,7 @@
         <x:v>pal_094</x:v>
       </x:c>
       <x:c r="B95" s="3" t="str">
-        <x:v>海誓龙</x:v>
+        <x:v>海棠水鹿</x:v>
       </x:c>
       <x:c r="C95" s="3" t="str">
         <x:v>草、水</x:v>
@@ -5059,7 +5059,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F95" s="3" t="str">
-        <x:v>night_base, elem_草, elem_水, role_治疗, tier_pT2, role_水系牵制</x:v>
+        <x:v>night_base, elem_草, elem_水, role_治疗, tier_pT2, role_水系牵制, shop_store_50, shop_store_68</x:v>
       </x:c>
       <x:c r="G95" s="3" t="str">
         <x:v>40</x:v>
@@ -5094,7 +5094,7 @@
         <x:v>pal_095</x:v>
       </x:c>
       <x:c r="B96" s="3" t="str">
-        <x:v>花丽娜</x:v>
+        <x:v>百花灵鹿</x:v>
       </x:c>
       <x:c r="C96" s="3" t="str">
         <x:v>草</x:v>
@@ -5106,7 +5106,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F96" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT2, role_远点压制, shop_store_50</x:v>
       </x:c>
       <x:c r="G96" s="3" t="str">
         <x:v>25</x:v>
@@ -5141,7 +5141,7 @@
         <x:v>pal_096</x:v>
       </x:c>
       <x:c r="B97" s="3" t="str">
-        <x:v>熔岩兽</x:v>
+        <x:v>熔岩巨兽</x:v>
       </x:c>
       <x:c r="C97" s="3" t="str">
         <x:v>火、地</x:v>
@@ -5153,7 +5153,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F97" s="3" t="str">
-        <x:v>night_base, elem_火, elem_地, role_坦克, tier_pT2, role_重甲抗压</x:v>
+        <x:v>night_base, elem_火, elem_地, role_坦克, tier_pT2, role_重甲抗压, shop_store_69</x:v>
       </x:c>
       <x:c r="G97" s="3" t="str">
         <x:v>50</x:v>
@@ -5188,7 +5188,7 @@
         <x:v>pal_097</x:v>
       </x:c>
       <x:c r="B98" s="3" t="str">
-        <x:v>寒霜兽</x:v>
+        <x:v>寒岩巨兽</x:v>
       </x:c>
       <x:c r="C98" s="3" t="str">
         <x:v>冰、地</x:v>
@@ -5200,7 +5200,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F98" s="3" t="str">
-        <x:v>night_base, elem_冰, elem_地, role_坦克, tier_pT2, role_重甲抗压</x:v>
+        <x:v>night_base, elem_冰, elem_地, role_坦克, tier_pT2, role_重甲抗压, shop_store_51, shop_store_69</x:v>
       </x:c>
       <x:c r="G98" s="3" t="str">
         <x:v>40</x:v>
@@ -5235,7 +5235,7 @@
         <x:v>pal_098</x:v>
       </x:c>
       <x:c r="B99" s="3" t="str">
-        <x:v>君王美露帕</x:v>
+        <x:v>云顶巨驼</x:v>
       </x:c>
       <x:c r="C99" s="3" t="str">
         <x:v>无</x:v>
@@ -5247,7 +5247,7 @@
         <x:v>经济</x:v>
       </x:c>
       <x:c r="F99" s="3" t="str">
-        <x:v>night_base, elem_无, role_经济, tier_pT2, role_夹击牵制</x:v>
+        <x:v>night_base, elem_无, role_经济, tier_pT2, role_夹击牵制, shop_store_51, shop_store_69</x:v>
       </x:c>
       <x:c r="G99" s="3" t="str">
         <x:v>35</x:v>
@@ -5282,7 +5282,7 @@
         <x:v>pal_099</x:v>
       </x:c>
       <x:c r="B100" s="3" t="str">
-        <x:v>冰帝美露帕</x:v>
+        <x:v>冰峰巨驼</x:v>
       </x:c>
       <x:c r="C100" s="3" t="str">
         <x:v>冰</x:v>
@@ -5294,7 +5294,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F100" s="3" t="str">
-        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_抗压承伤, shop_store_51, shop_store_69</x:v>
       </x:c>
       <x:c r="G100" s="3" t="str">
         <x:v>15</x:v>
@@ -5329,7 +5329,7 @@
         <x:v>pal_100</x:v>
       </x:c>
       <x:c r="B101" s="3" t="str">
-        <x:v>森猛犸</x:v>
+        <x:v>青林巨象</x:v>
       </x:c>
       <x:c r="C101" s="3" t="str">
         <x:v>草</x:v>
@@ -5341,7 +5341,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F101" s="3" t="str">
-        <x:v>night_base, elem_草, role_坦克, tier_pT2, role_重甲抗压</x:v>
+        <x:v>night_base, elem_草, role_坦克, tier_pT2, role_重甲抗压, shop_store_51, shop_store_69</x:v>
       </x:c>
       <x:c r="G101" s="3" t="str">
         <x:v>50</x:v>
@@ -5376,7 +5376,7 @@
         <x:v>pal_101</x:v>
       </x:c>
       <x:c r="B102" s="3" t="str">
-        <x:v>雪猛犸</x:v>
+        <x:v>白牙雪象</x:v>
       </x:c>
       <x:c r="C102" s="3" t="str">
         <x:v>冰</x:v>
@@ -5388,7 +5388,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F102" s="3" t="str">
-        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_重甲抗压</x:v>
+        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_重甲抗压, shop_store_51, shop_store_69</x:v>
       </x:c>
       <x:c r="G102" s="3" t="str">
         <x:v>35</x:v>
@@ -5423,7 +5423,7 @@
         <x:v>pal_102</x:v>
       </x:c>
       <x:c r="B103" s="3" t="str">
-        <x:v>白绒雪怪</x:v>
+        <x:v>白绒雪猿</x:v>
       </x:c>
       <x:c r="C103" s="3" t="str">
         <x:v>冰</x:v>
@@ -5435,7 +5435,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F103" s="3" t="str">
-        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_冰, role_坦克, tier_pT2, role_抗压承伤, elite_high, shop_store_51</x:v>
       </x:c>
       <x:c r="G103" s="3" t="str">
         <x:v>15</x:v>
@@ -5470,7 +5470,7 @@
         <x:v>pal_103</x:v>
       </x:c>
       <x:c r="B104" s="3" t="str">
-        <x:v>绿苔绒怪</x:v>
+        <x:v>绿苔巨猿</x:v>
       </x:c>
       <x:c r="C104" s="3" t="str">
         <x:v>草</x:v>
@@ -5482,7 +5482,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F104" s="3" t="str">
-        <x:v>night_base, elem_草, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_草, role_坦克, tier_pT2, role_抗压承伤, elite_high, shop_store_70</x:v>
       </x:c>
       <x:c r="G104" s="3" t="str">
         <x:v>15</x:v>
@@ -5517,7 +5517,7 @@
         <x:v>pal_104</x:v>
       </x:c>
       <x:c r="B105" s="3" t="str">
-        <x:v>铠格力斯</x:v>
+        <x:v>铁甲巨兕</x:v>
       </x:c>
       <x:c r="C105" s="3" t="str">
         <x:v>地、草</x:v>
@@ -5529,7 +5529,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F105" s="3" t="str">
-        <x:v>night_base, elem_地, elem_草, role_坦克, tier_pT2, role_抗压承伤</x:v>
+        <x:v>night_base, elem_地, elem_草, role_坦克, tier_pT2, role_抗压承伤, elite_high, shop_store_52, shop_store_70</x:v>
       </x:c>
       <x:c r="G105" s="3" t="str">
         <x:v>15</x:v>
@@ -5564,7 +5564,7 @@
         <x:v>pal_105</x:v>
       </x:c>
       <x:c r="B106" s="3" t="str">
-        <x:v>云海鹿</x:v>
+        <x:v>云海白鹿</x:v>
       </x:c>
       <x:c r="C106" s="3" t="str">
         <x:v>无</x:v>
@@ -5576,7 +5576,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F106" s="3" t="str">
-        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制</x:v>
+        <x:v>night_base, elem_无, role_机动, tier_pT2, role_机动压制, elite_high, shop_store_52, shop_store_70</x:v>
       </x:c>
       <x:c r="G106" s="3" t="str">
         <x:v>10</x:v>
@@ -5611,7 +5611,7 @@
         <x:v>pal_106</x:v>
       </x:c>
       <x:c r="B107" s="3" t="str">
-        <x:v>夜幕魔蝠</x:v>
+        <x:v>夜幕巨蝠</x:v>
       </x:c>
       <x:c r="C107" s="3" t="str">
         <x:v>暗</x:v>
@@ -5623,7 +5623,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F107" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_召唤铺场</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT2, role_召唤铺场, elite_high, shop_store_52, shop_store_70</x:v>
       </x:c>
       <x:c r="G107" s="3" t="str">
         <x:v>35</x:v>
@@ -5658,7 +5658,7 @@
         <x:v>pal_107</x:v>
       </x:c>
       <x:c r="B108" s="3" t="str">
-        <x:v>天羽龙</x:v>
+        <x:v>天羽云螭</x:v>
       </x:c>
       <x:c r="C108" s="3" t="str">
         <x:v>龙</x:v>
@@ -5670,7 +5670,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F108" s="3" t="str">
-        <x:v>night_base, elem_龙, role_机动, tier_pT2, role_机动压制</x:v>
+        <x:v>night_base, elem_龙, role_机动, tier_pT2, role_机动压制, elite_high, shop_store_52, shop_store_70</x:v>
       </x:c>
       <x:c r="G108" s="3" t="str">
         <x:v>70</x:v>
@@ -5705,7 +5705,7 @@
         <x:v>pal_108</x:v>
       </x:c>
       <x:c r="B109" s="3" t="str">
-        <x:v>焰煌</x:v>
+        <x:v>焰羽赤雕</x:v>
       </x:c>
       <x:c r="C109" s="3" t="str">
         <x:v>火</x:v>
@@ -5717,7 +5717,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F109" s="3" t="str">
-        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系重压</x:v>
+        <x:v>night_base, elem_火, role_输出, tier_pT2, role_火系重压, shop_store_52, shop_store_70</x:v>
       </x:c>
       <x:c r="G109" s="3" t="str">
         <x:v>60</x:v>
@@ -5752,7 +5752,7 @@
         <x:v>pal_109</x:v>
       </x:c>
       <x:c r="B110" s="3" t="str">
-        <x:v>雷冥鸟</x:v>
+        <x:v>冥羽黑乌</x:v>
       </x:c>
       <x:c r="C110" s="3" t="str">
         <x:v>暗</x:v>
@@ -5764,7 +5764,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F110" s="3" t="str">
-        <x:v>night_base, elem_暗, role_机动, tier_pT2, role_土系抗压</x:v>
+        <x:v>night_base, elem_暗, role_机动, tier_pT2, role_土系抗压, shop_store_52</x:v>
       </x:c>
       <x:c r="G110" s="3" t="str">
         <x:v>10</x:v>
@@ -5799,7 +5799,7 @@
         <x:v>pal_110</x:v>
       </x:c>
       <x:c r="B111" s="3" t="str">
-        <x:v>魔渊龙</x:v>
+        <x:v>渊鳞黑蛟</x:v>
       </x:c>
       <x:c r="C111" s="3" t="str">
         <x:v>龙、暗</x:v>
@@ -5811,7 +5811,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F111" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_暗, role_坦克, tier_pT2, role_诅咒牵制</x:v>
+        <x:v>night_base, elem_龙, elem_暗, role_坦克, tier_pT2, role_诅咒牵制, shop_store_71</x:v>
       </x:c>
       <x:c r="G111" s="3" t="str">
         <x:v>50</x:v>
@@ -5846,7 +5846,7 @@
         <x:v>pal_111</x:v>
       </x:c>
       <x:c r="B112" s="3" t="str">
-        <x:v>冥铠蝎</x:v>
+        <x:v>毒甲蝎将</x:v>
       </x:c>
       <x:c r="C112" s="3" t="str">
         <x:v>暗、地</x:v>
@@ -5858,7 +5858,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F112" s="3" t="str">
-        <x:v>night_base, elem_暗, elem_地, role_坦克, tier_pT3, role_抗压承伤</x:v>
+        <x:v>night_base, elem_暗, elem_地, role_坦克, tier_pT3, role_抗压承伤, shop_store_53, shop_store_71</x:v>
       </x:c>
       <x:c r="G112" s="3" t="str">
         <x:v>20</x:v>
@@ -5893,7 +5893,7 @@
         <x:v>pal_112</x:v>
       </x:c>
       <x:c r="B113" s="3" t="str">
-        <x:v>阿努比斯</x:v>
+        <x:v>石猿战将</x:v>
       </x:c>
       <x:c r="C113" s="3" t="str">
         <x:v>地</x:v>
@@ -5905,7 +5905,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F113" s="3" t="str">
-        <x:v>night_base, elem_地, role_输出, tier_pT3, role_土系抗压</x:v>
+        <x:v>night_base, elem_地, role_输出, tier_pT3, role_土系抗压, special_merchant, shop_store_53, shop_store_71</x:v>
       </x:c>
       <x:c r="G113" s="3" t="str">
         <x:v>50</x:v>
@@ -5940,7 +5940,7 @@
         <x:v>pal_113</x:v>
       </x:c>
       <x:c r="B114" s="3" t="str">
-        <x:v>覆海龙</x:v>
+        <x:v>覆海蛟王</x:v>
       </x:c>
       <x:c r="C114" s="3" t="str">
         <x:v>龙、水</x:v>
@@ -5952,7 +5952,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F114" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_水, role_治疗, tier_pT3, role_水系牵制</x:v>
+        <x:v>night_base, elem_龙, elem_水, role_治疗, tier_pT3, role_水系牵制, special_merchant, shop_store_53, shop_store_71</x:v>
       </x:c>
       <x:c r="G114" s="3" t="str">
         <x:v>50</x:v>
@@ -5987,7 +5987,7 @@
         <x:v>pal_114</x:v>
       </x:c>
       <x:c r="B115" s="3" t="str">
-        <x:v>腾炎龙</x:v>
+        <x:v>赤焰龙君</x:v>
       </x:c>
       <x:c r="C115" s="3" t="str">
         <x:v>龙、火</x:v>
@@ -5999,7 +5999,7 @@
         <x:v>输出</x:v>
       </x:c>
       <x:c r="F115" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_火, role_输出, tier_pT3, role_火系重压</x:v>
+        <x:v>night_base, elem_龙, elem_火, role_输出, tier_pT3, role_火系重压, special_merchant, shop_store_53, shop_store_71</x:v>
       </x:c>
       <x:c r="G115" s="3" t="str">
         <x:v>60</x:v>
@@ -6034,7 +6034,7 @@
         <x:v>pal_115</x:v>
       </x:c>
       <x:c r="B116" s="3" t="str">
-        <x:v>朱雀</x:v>
+        <x:v>南明朱雀</x:v>
       </x:c>
       <x:c r="C116" s="3" t="str">
         <x:v>火</x:v>
@@ -6046,7 +6046,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F116" s="3" t="str">
-        <x:v>night_base, elem_火, role_机动, tier_pT3, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_机动, tier_pT3, role_火系压制, special_merchant, shop_store_53, shop_store_71</x:v>
       </x:c>
       <x:c r="G116" s="3" t="str">
         <x:v>25</x:v>
@@ -6081,7 +6081,7 @@
         <x:v>pal_116</x:v>
       </x:c>
       <x:c r="B117" s="3" t="str">
-        <x:v>清雀</x:v>
+        <x:v>净瓶青鸾</x:v>
       </x:c>
       <x:c r="C117" s="3" t="str">
         <x:v>水</x:v>
@@ -6093,7 +6093,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F117" s="3" t="str">
-        <x:v>night_base, elem_水, role_治疗, tier_pT3, role_水系牵制</x:v>
+        <x:v>night_base, elem_水, role_治疗, tier_pT3, role_水系牵制, special_merchant, shop_store_53</x:v>
       </x:c>
       <x:c r="G117" s="3" t="str">
         <x:v>50</x:v>
@@ -6128,7 +6128,7 @@
         <x:v>pal_117</x:v>
       </x:c>
       <x:c r="B118" s="3" t="str">
-        <x:v>暴电熊</x:v>
+        <x:v>九霄熊王</x:v>
       </x:c>
       <x:c r="C118" s="3" t="str">
         <x:v>雷</x:v>
@@ -6140,7 +6140,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F118" s="3" t="str">
-        <x:v>night_base, elem_雷, role_控制, tier_pT3, role_风系牵制</x:v>
+        <x:v>night_base, elem_雷, role_控制, tier_pT3, role_风系牵制, special_merchant, shop_store_72</x:v>
       </x:c>
       <x:c r="G118" s="3" t="str">
         <x:v>30</x:v>
@@ -6175,7 +6175,7 @@
         <x:v>pal_118</x:v>
       </x:c>
       <x:c r="B119" s="3" t="str">
-        <x:v>百合女王</x:v>
+        <x:v>百花鹿仙</x:v>
       </x:c>
       <x:c r="C119" s="3" t="str">
         <x:v>草</x:v>
@@ -6187,7 +6187,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F119" s="3" t="str">
-        <x:v>night_base, elem_草, role_治疗, tier_pT3, role_远点压制</x:v>
+        <x:v>night_base, elem_草, role_治疗, tier_pT3, role_远点压制, shop_store_54, shop_store_72</x:v>
       </x:c>
       <x:c r="G119" s="3" t="str">
         <x:v>50</x:v>
@@ -6222,7 +6222,7 @@
         <x:v>pal_119</x:v>
       </x:c>
       <x:c r="B120" s="3" t="str">
-        <x:v>黑月女王</x:v>
+        <x:v>黑月狐姬</x:v>
       </x:c>
       <x:c r="C120" s="3" t="str">
         <x:v>暗</x:v>
@@ -6234,7 +6234,7 @@
         <x:v>治疗</x:v>
       </x:c>
       <x:c r="F120" s="3" t="str">
-        <x:v>night_base, elem_暗, role_治疗, tier_pT3, role_土系抗压</x:v>
+        <x:v>night_base, elem_暗, role_治疗, tier_pT3, role_土系抗压, shop_store_54, shop_store_72</x:v>
       </x:c>
       <x:c r="G120" s="3" t="str">
         <x:v>50</x:v>
@@ -6269,7 +6269,7 @@
         <x:v>pal_120</x:v>
       </x:c>
       <x:c r="B121" s="3" t="str">
-        <x:v>荷鲁斯</x:v>
+        <x:v>火云鹏王</x:v>
       </x:c>
       <x:c r="C121" s="3" t="str">
         <x:v>火</x:v>
@@ -6281,7 +6281,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F121" s="3" t="str">
-        <x:v>night_base, elem_火, role_机动, tier_pT3, role_火系压制</x:v>
+        <x:v>night_base, elem_火, role_机动, tier_pT3, role_火系压制, shop_store_54, shop_store_72</x:v>
       </x:c>
       <x:c r="G121" s="3" t="str">
         <x:v>25</x:v>
@@ -6316,7 +6316,7 @@
         <x:v>pal_121</x:v>
       </x:c>
       <x:c r="B122" s="3" t="str">
-        <x:v>波鲁杰克斯</x:v>
+        <x:v>雷泽龙王</x:v>
       </x:c>
       <x:c r="C122" s="3" t="str">
         <x:v>龙、雷</x:v>
@@ -6328,7 +6328,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F122" s="3" t="str">
-        <x:v>night_base, elem_龙, elem_雷, role_控制, tier_pT3, role_风系牵制</x:v>
+        <x:v>night_base, elem_龙, elem_雷, role_控制, tier_pT3, role_风系牵制, shop_store_54, shop_store_72</x:v>
       </x:c>
       <x:c r="G122" s="3" t="str">
         <x:v>60</x:v>
@@ -6363,7 +6363,7 @@
         <x:v>pal_122</x:v>
       </x:c>
       <x:c r="B123" s="3" t="str">
-        <x:v>异构格里芬</x:v>
+        <x:v>玄羽雕尊</x:v>
       </x:c>
       <x:c r="C123" s="3" t="str">
         <x:v>暗</x:v>
@@ -6375,7 +6375,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F123" s="3" t="str">
-        <x:v>night_base, elem_暗, role_机动, tier_pT3, role_土系抗压</x:v>
+        <x:v>night_base, elem_暗, role_机动, tier_pT3, role_土系抗压, shop_store_54, shop_store_72</x:v>
       </x:c>
       <x:c r="G123" s="3" t="str">
         <x:v>25</x:v>
@@ -6410,7 +6410,7 @@
         <x:v>pal_123</x:v>
       </x:c>
       <x:c r="B124" s="3" t="str">
-        <x:v>圣光骑士</x:v>
+        <x:v>白象护法</x:v>
       </x:c>
       <x:c r="C124" s="3" t="str">
         <x:v>无</x:v>
@@ -6422,7 +6422,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F124" s="3" t="str">
-        <x:v>night_base, elem_无, role_坦克, tier_pT3, role_重甲抗压</x:v>
+        <x:v>night_base, elem_无, role_坦克, tier_pT3, role_重甲抗压, shop_store_54</x:v>
       </x:c>
       <x:c r="G124" s="3" t="str">
         <x:v>70</x:v>
@@ -6457,7 +6457,7 @@
         <x:v>pal_124</x:v>
       </x:c>
       <x:c r="B125" s="3" t="str">
-        <x:v>混沌骑士</x:v>
+        <x:v>混世魔猿</x:v>
       </x:c>
       <x:c r="C125" s="3" t="str">
         <x:v>暗</x:v>
@@ -6469,7 +6469,7 @@
         <x:v>坦克</x:v>
       </x:c>
       <x:c r="F125" s="3" t="str">
-        <x:v>night_base, elem_暗, role_坦克, tier_pT3, role_重甲抗压</x:v>
+        <x:v>night_base, elem_暗, role_坦克, tier_pT3, role_重甲抗压, shop_store_73</x:v>
       </x:c>
       <x:c r="G125" s="3" t="str">
         <x:v>60</x:v>
@@ -6504,7 +6504,7 @@
         <x:v>pal_125</x:v>
       </x:c>
       <x:c r="B126" s="3" t="str">
-        <x:v>唤冬兽</x:v>
+        <x:v>寒狮妖王</x:v>
       </x:c>
       <x:c r="C126" s="3" t="str">
         <x:v>冰</x:v>
@@ -6516,7 +6516,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F126" s="3" t="str">
-        <x:v>night_base, elem_冰, role_控制, tier_pT3, role_水系牵制</x:v>
+        <x:v>night_base, elem_冰, role_控制, tier_pT3, role_水系牵制, shop_store_55, shop_store_73</x:v>
       </x:c>
       <x:c r="G126" s="3" t="str">
         <x:v>60</x:v>
@@ -6551,7 +6551,7 @@
         <x:v>pal_126</x:v>
       </x:c>
       <x:c r="B127" s="3" t="str">
-        <x:v>唤夜兽</x:v>
+        <x:v>幽冥獒王</x:v>
       </x:c>
       <x:c r="C127" s="3" t="str">
         <x:v>暗</x:v>
@@ -6563,7 +6563,7 @@
         <x:v>控制</x:v>
       </x:c>
       <x:c r="F127" s="3" t="str">
-        <x:v>night_base, elem_暗, role_控制, tier_pT3, role_土系抗压</x:v>
+        <x:v>night_base, elem_暗, role_控制, tier_pT3, role_土系抗压, shop_store_37, shop_store_55, shop_store_73</x:v>
       </x:c>
       <x:c r="G127" s="3" t="str">
         <x:v>60</x:v>
@@ -6598,7 +6598,7 @@
         <x:v>pal_127</x:v>
       </x:c>
       <x:c r="B128" s="3" t="str">
-        <x:v>空涡龙</x:v>
+        <x:v>九天龙君</x:v>
       </x:c>
       <x:c r="C128" s="3" t="str">
         <x:v>龙</x:v>
@@ -6610,7 +6610,7 @@
         <x:v>机动</x:v>
       </x:c>
       <x:c r="F128" s="3" t="str">
-        <x:v>night_base, elem_龙, role_机动, tier_pT3, role_机动压制</x:v>
+        <x:v>night_base, elem_龙, role_机动, tier_pT3, role_机动压制, shop_store_37, shop_store_55, shop_store_73</x:v>
       </x:c>
       <x:c r="G128" s="3" t="str">
         <x:v>50</x:v>
@@ -6649,7 +6649,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3be4c4067e704147"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf328001719194137"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6659,7 +6659,7 @@
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" customWidth="1"/>
-    <x:col min="2" max="2" width="10" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" customWidth="1"/>
     <x:col min="4" max="4" width="22" customWidth="1"/>
     <x:col min="5" max="5" width="15" customWidth="1"/>
@@ -6703,7 +6703,7 @@
         <x:v>night_base</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>夜市商人</x:v>
+        <x:v>寅将军</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
         <x:v>通用店</x:v>
@@ -6729,16 +6729,16 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>elem_无</x:v>
+        <x:v>elem_火</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>无系商品店</x:v>
+        <x:v>熊山君</x:v>
       </x:c>
       <x:c r="C3" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>元素, 无</x:v>
+        <x:v>元素, 火</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
         <x:v>10</x:v>
@@ -6753,21 +6753,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>出售无元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售火元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="str">
-        <x:v>elem_火</x:v>
+        <x:v>elem_水</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>火系商品店</x:v>
+        <x:v>特处士</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D4" s="3" t="str">
-        <x:v>元素, 火</x:v>
+        <x:v>元素, 水</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
         <x:v>10</x:v>
@@ -6782,21 +6782,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>出售火元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售水元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>elem_水</x:v>
+        <x:v>elem_草</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>水系商品店</x:v>
+        <x:v>刘伯钦</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>元素, 水</x:v>
+        <x:v>元素, 草</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>10</x:v>
@@ -6811,21 +6811,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
-        <x:v>出售水元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售草元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
-        <x:v>elem_草</x:v>
+        <x:v>elem_雷</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>草系商品店</x:v>
+        <x:v>孙悟空</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>元素, 草</x:v>
+        <x:v>元素, 雷</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
         <x:v>10</x:v>
@@ -6840,21 +6840,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
-        <x:v>出售草元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售雷元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="str">
-        <x:v>elem_雷</x:v>
+        <x:v>elem_冰</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>雷系商品店</x:v>
+        <x:v>小白龙</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>元素, 雷</x:v>
+        <x:v>元素, 冰</x:v>
       </x:c>
       <x:c r="E7" s="3" t="str">
         <x:v>10</x:v>
@@ -6869,21 +6869,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
-        <x:v>出售雷元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售冰元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="str">
-        <x:v>elem_冰</x:v>
+        <x:v>elem_地</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>冰系商品店</x:v>
+        <x:v>金池长老</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D8" s="3" t="str">
-        <x:v>元素, 冰</x:v>
+        <x:v>元素, 地</x:v>
       </x:c>
       <x:c r="E8" s="3" t="str">
         <x:v>10</x:v>
@@ -6898,21 +6898,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>出售冰元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售地元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="str">
-        <x:v>elem_地</x:v>
+        <x:v>elem_暗</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>地系商品店</x:v>
+        <x:v>黑熊精</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>元素, 地</x:v>
+        <x:v>元素, 暗</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
         <x:v>10</x:v>
@@ -6927,21 +6927,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>出售地元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售暗元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="3" t="str">
-        <x:v>elem_暗</x:v>
+        <x:v>elem_龙</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>暗系商品店</x:v>
+        <x:v>凌虚子</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
         <x:v>元素店</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str">
-        <x:v>元素, 暗</x:v>
+        <x:v>元素, 龙</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
         <x:v>10</x:v>
@@ -6956,27 +6956,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>出售暗元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售龙元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="3" t="str">
-        <x:v>elem_龙</x:v>
+        <x:v>role_召唤</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>龙系商品店</x:v>
+        <x:v>苍狼精</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>元素店</x:v>
+        <x:v>定位店</x:v>
       </x:c>
       <x:c r="D11" s="3" t="str">
-        <x:v>元素, 龙</x:v>
+        <x:v>定位, 召唤</x:v>
       </x:c>
       <x:c r="E11" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
         <x:v>标准价格</x:v>
@@ -6985,21 +6985,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>出售龙元素宠物；双属性宠物同时进入两个对应元素店。</x:v>
+        <x:v>出售召唤定位宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="3" t="str">
-        <x:v>role_召唤</x:v>
+        <x:v>role_召唤铺场</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>召唤商品店</x:v>
+        <x:v>猪八戒</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>定位, 召唤</x:v>
+        <x:v>定位, 召唤铺场</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
         <x:v>10</x:v>
@@ -7014,21 +7014,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>出售召唤定位宠物。</x:v>
+        <x:v>出售召唤铺场倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="3" t="str">
-        <x:v>role_召唤铺场</x:v>
+        <x:v>role_坦克</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
-        <x:v>召唤铺场商品店</x:v>
+        <x:v>黄风怪</x:v>
       </x:c>
       <x:c r="C13" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D13" s="3" t="str">
-        <x:v>定位, 召唤铺场</x:v>
+        <x:v>定位, 坦克</x:v>
       </x:c>
       <x:c r="E13" s="3" t="str">
         <x:v>10</x:v>
@@ -7043,27 +7043,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>出售召唤铺场倾向宠物。</x:v>
+        <x:v>出售坦克/前排宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="3" t="str">
-        <x:v>role_坦克</x:v>
+        <x:v>role_控制</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>前排商品店</x:v>
+        <x:v>灵吉菩萨</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>定位, 坦克</x:v>
+        <x:v>定位, 控制</x:v>
       </x:c>
       <x:c r="E14" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="3" t="str">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
         <x:v>标准价格</x:v>
@@ -7072,27 +7072,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
-        <x:v>出售坦克/前排宠物。</x:v>
+        <x:v>出售控制定位宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="3" t="str">
-        <x:v>role_控制</x:v>
+        <x:v>role_治疗</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>控制商品店</x:v>
+        <x:v>沙悟净</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>定位, 控制</x:v>
+        <x:v>定位, 治疗</x:v>
       </x:c>
       <x:c r="E15" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="3" t="str">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
         <x:v>标准价格</x:v>
@@ -7101,27 +7101,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
-        <x:v>出售控制定位宠物。</x:v>
+        <x:v>出售治疗定位宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="3" t="str">
-        <x:v>role_治疗</x:v>
+        <x:v>role_输出</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>治疗商品店</x:v>
+        <x:v>沙僧</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D16" s="3" t="str">
-        <x:v>定位, 治疗</x:v>
+        <x:v>定位, 输出</x:v>
       </x:c>
       <x:c r="E16" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F16" s="3" t="str">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G16" s="3" t="str">
         <x:v>标准价格</x:v>
@@ -7130,27 +7130,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
-        <x:v>出售治疗定位宠物。</x:v>
+        <x:v>出售输出定位宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="3" t="str">
-        <x:v>role_输出</x:v>
+        <x:v>role_经济</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>输出商品店</x:v>
+        <x:v>黎山老母</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D17" s="3" t="str">
-        <x:v>定位, 输出</x:v>
+        <x:v>定位, 经济</x:v>
       </x:c>
       <x:c r="E17" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F17" s="3" t="str">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
         <x:v>标准价格</x:v>
@@ -7159,27 +7159,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>出售输出定位宠物。</x:v>
+        <x:v>出售经济定位宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="3" t="str">
-        <x:v>role_经济</x:v>
+        <x:v>role_机动</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>经济商品店</x:v>
+        <x:v>观音</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D18" s="3" t="str">
-        <x:v>定位, 经济</x:v>
+        <x:v>定位, 机动</x:v>
       </x:c>
       <x:c r="E18" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="3" t="str">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
         <x:v>标准价格</x:v>
@@ -7188,21 +7188,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>出售经济定位宠物。</x:v>
+        <x:v>出售机动定位宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="3" t="str">
-        <x:v>role_机动</x:v>
+        <x:v>role_机动压制</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>机动商品店</x:v>
+        <x:v>普贤</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D19" s="3" t="str">
-        <x:v>定位, 机动</x:v>
+        <x:v>定位, 机动压制</x:v>
       </x:c>
       <x:c r="E19" s="3" t="str">
         <x:v>10</x:v>
@@ -7217,21 +7217,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>出售机动定位宠物。</x:v>
+        <x:v>出售机动压制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="3" t="str">
-        <x:v>role_机动压制</x:v>
+        <x:v>role_抗压承伤</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
-        <x:v>机动压制商品店</x:v>
+        <x:v>文殊</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D20" s="3" t="str">
-        <x:v>定位, 机动压制</x:v>
+        <x:v>定位, 抗压承伤</x:v>
       </x:c>
       <x:c r="E20" s="3" t="str">
         <x:v>10</x:v>
@@ -7246,21 +7246,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>出售机动压制倾向宠物。</x:v>
+        <x:v>出售抗压承伤倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="3" t="str">
-        <x:v>role_抗压承伤</x:v>
+        <x:v>role_重甲抗压</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
-        <x:v>抗压承伤商品店</x:v>
+        <x:v>镇元大仙</x:v>
       </x:c>
       <x:c r="C21" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D21" s="3" t="str">
-        <x:v>定位, 抗压承伤</x:v>
+        <x:v>定位, 重甲抗压</x:v>
       </x:c>
       <x:c r="E21" s="3" t="str">
         <x:v>10</x:v>
@@ -7275,21 +7275,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>出售抗压承伤倾向宠物。</x:v>
+        <x:v>出售重甲抗压倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="3" t="str">
-        <x:v>role_重甲抗压</x:v>
+        <x:v>role_远点压制</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
-        <x:v>重甲抗压商品店</x:v>
+        <x:v>观音菩萨</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D22" s="3" t="str">
-        <x:v>定位, 重甲抗压</x:v>
+        <x:v>定位, 远点压制</x:v>
       </x:c>
       <x:c r="E22" s="3" t="str">
         <x:v>10</x:v>
@@ -7304,21 +7304,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>出售重甲抗压倾向宠物。</x:v>
+        <x:v>出售远点压制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="3" t="str">
-        <x:v>role_远点压制</x:v>
+        <x:v>role_风系铺场</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
-        <x:v>远点压制商品店</x:v>
+        <x:v>白骨精</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D23" s="3" t="str">
-        <x:v>定位, 远点压制</x:v>
+        <x:v>定位, 风系铺场</x:v>
       </x:c>
       <x:c r="E23" s="3" t="str">
         <x:v>10</x:v>
@@ -7333,21 +7333,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
-        <x:v>出售远点压制倾向宠物。</x:v>
+        <x:v>出售风系铺场倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="3" t="str">
-        <x:v>role_风系铺场</x:v>
+        <x:v>role_风系牵制</x:v>
       </x:c>
       <x:c r="B24" s="3" t="str">
-        <x:v>风系铺场商品店</x:v>
+        <x:v>黄袍怪</x:v>
       </x:c>
       <x:c r="C24" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D24" s="3" t="str">
-        <x:v>定位, 风系铺场</x:v>
+        <x:v>定位, 风系牵制</x:v>
       </x:c>
       <x:c r="E24" s="3" t="str">
         <x:v>10</x:v>
@@ -7362,21 +7362,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>出售风系铺场倾向宠物。</x:v>
+        <x:v>出售风系牵制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="3" t="str">
-        <x:v>role_风系牵制</x:v>
+        <x:v>role_火系压制</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
-        <x:v>风系牵制商品店</x:v>
+        <x:v>百花羞</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D25" s="3" t="str">
-        <x:v>定位, 风系牵制</x:v>
+        <x:v>定位, 火系压制</x:v>
       </x:c>
       <x:c r="E25" s="3" t="str">
         <x:v>10</x:v>
@@ -7391,21 +7391,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>出售风系牵制倾向宠物。</x:v>
+        <x:v>出售火系压制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="3" t="str">
-        <x:v>role_火系压制</x:v>
+        <x:v>role_火系重压</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>火系压制商品店</x:v>
+        <x:v>宝象国国王</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D26" s="3" t="str">
-        <x:v>定位, 火系压制</x:v>
+        <x:v>定位, 火系重压</x:v>
       </x:c>
       <x:c r="E26" s="3" t="str">
         <x:v>10</x:v>
@@ -7420,21 +7420,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>出售火系压制倾向宠物。</x:v>
+        <x:v>出售火系重压倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="3" t="str">
-        <x:v>role_火系重压</x:v>
+        <x:v>role_水系控场</x:v>
       </x:c>
       <x:c r="B27" s="3" t="str">
-        <x:v>火系重压商品店</x:v>
+        <x:v>金角大王</x:v>
       </x:c>
       <x:c r="C27" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D27" s="3" t="str">
-        <x:v>定位, 火系重压</x:v>
+        <x:v>定位, 水系控场</x:v>
       </x:c>
       <x:c r="E27" s="3" t="str">
         <x:v>10</x:v>
@@ -7449,21 +7449,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
-        <x:v>出售火系重压倾向宠物。</x:v>
+        <x:v>出售水系控场倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="3" t="str">
-        <x:v>role_水系控场</x:v>
+        <x:v>role_水系牵制</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>水系控场商品店</x:v>
+        <x:v>银角大王</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
-        <x:v>定位, 水系控场</x:v>
+        <x:v>定位, 水系牵制</x:v>
       </x:c>
       <x:c r="E28" s="3" t="str">
         <x:v>10</x:v>
@@ -7478,21 +7478,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>出售水系控场倾向宠物。</x:v>
+        <x:v>出售水系牵制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="3" t="str">
-        <x:v>role_水系牵制</x:v>
+        <x:v>role_土系抗压</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
-        <x:v>水系牵制商品店</x:v>
+        <x:v>九尾狐</x:v>
       </x:c>
       <x:c r="C29" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D29" s="3" t="str">
-        <x:v>定位, 水系牵制</x:v>
+        <x:v>定位, 土系抗压</x:v>
       </x:c>
       <x:c r="E29" s="3" t="str">
         <x:v>10</x:v>
@@ -7507,21 +7507,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
-        <x:v>出售水系牵制倾向宠物。</x:v>
+        <x:v>出售土系抗压倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="3" t="str">
-        <x:v>role_土系抗压</x:v>
+        <x:v>role_夹击牵制</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>土系抗压商品店</x:v>
+        <x:v>狐阿七</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D30" s="3" t="str">
-        <x:v>定位, 土系抗压</x:v>
+        <x:v>定位, 夹击牵制</x:v>
       </x:c>
       <x:c r="E30" s="3" t="str">
         <x:v>10</x:v>
@@ -7536,21 +7536,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>出售土系抗压倾向宠物。</x:v>
+        <x:v>出售夹击牵制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="3" t="str">
-        <x:v>role_夹击牵制</x:v>
+        <x:v>role_成长输出</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>夹击牵制商品店</x:v>
+        <x:v>狮猁王</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D31" s="3" t="str">
-        <x:v>定位, 夹击牵制</x:v>
+        <x:v>定位, 成长输出</x:v>
       </x:c>
       <x:c r="E31" s="3" t="str">
         <x:v>10</x:v>
@@ -7565,21 +7565,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>出售夹击牵制倾向宠物。</x:v>
+        <x:v>出售成长输出倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="3" t="str">
-        <x:v>role_成长输出</x:v>
+        <x:v>role_诅咒牵制</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
-        <x:v>成长输出商品店</x:v>
+        <x:v>红孩儿</x:v>
       </x:c>
       <x:c r="C32" s="3" t="str">
         <x:v>定位店</x:v>
       </x:c>
       <x:c r="D32" s="3" t="str">
-        <x:v>定位, 成长输出</x:v>
+        <x:v>定位, 诅咒牵制</x:v>
       </x:c>
       <x:c r="E32" s="3" t="str">
         <x:v>10</x:v>
@@ -7594,21 +7594,21 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
-        <x:v>出售成长输出倾向宠物。</x:v>
+        <x:v>出售诅咒牵制倾向宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="3" t="str">
-        <x:v>role_诅咒牵制</x:v>
+        <x:v>tier_pT1</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
-        <x:v>诅咒牵制商品店</x:v>
+        <x:v>鼍龙</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
-        <x:v>定位店</x:v>
+        <x:v>品质店</x:v>
       </x:c>
       <x:c r="D33" s="3" t="str">
-        <x:v>定位, 诅咒牵制</x:v>
+        <x:v>品质, 青铜</x:v>
       </x:c>
       <x:c r="E33" s="3" t="str">
         <x:v>10</x:v>
@@ -7623,27 +7623,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
-        <x:v>出售诅咒牵制倾向宠物。</x:v>
+        <x:v>出售青铜池宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>tier_pT1</x:v>
+        <x:v>tier_pT2</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>青铜商品店</x:v>
+        <x:v>虎力大仙</x:v>
       </x:c>
       <x:c r="C34" t="str">
         <x:v>品质店</x:v>
       </x:c>
       <x:c r="D34" t="str">
-        <x:v>品质, 青铜</x:v>
+        <x:v>品质, 白银</x:v>
       </x:c>
       <x:c r="E34" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F34" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G34" t="str">
         <x:v>标准价格</x:v>
@@ -7652,27 +7652,27 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I34" t="str">
-        <x:v>出售青铜池宠物。</x:v>
+        <x:v>出售白银池宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>tier_pT2</x:v>
+        <x:v>tier_pT3</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>白银商品店</x:v>
+        <x:v>鹿力大仙</x:v>
       </x:c>
       <x:c r="C35" t="str">
         <x:v>品质店</x:v>
       </x:c>
       <x:c r="D35" t="str">
-        <x:v>品质, 白银</x:v>
+        <x:v>品质, 黄金</x:v>
       </x:c>
       <x:c r="E35" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F35" t="str">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G35" t="str">
         <x:v>标准价格</x:v>
@@ -7681,100 +7681,1318 @@
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I35" t="str">
-        <x:v>出售白银池宠物。</x:v>
+        <x:v>出售黄金池宠物。</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
-        <x:v>tier_pT3</x:v>
+        <x:v>special_merchant</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>黄金商品店</x:v>
+        <x:v>羊力大仙</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>品质店</x:v>
+        <x:v>特殊店</x:v>
       </x:c>
       <x:c r="D36" t="str">
-        <x:v>品质, 黄金</x:v>
+        <x:v>特殊, 构筑</x:v>
       </x:c>
       <x:c r="E36" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F36" t="str">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G36" t="str">
-        <x:v>标准价格</x:v>
+        <x:v>事件价格</x:v>
       </x:c>
       <x:c r="H36" t="str">
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I36" t="str">
-        <x:v>出售黄金池宠物。</x:v>
+        <x:v>复制、升阶等特殊构筑事件引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
-        <x:v>special_merchant</x:v>
+        <x:v>elite_high</x:v>
       </x:c>
       <x:c r="B37" t="str">
-        <x:v>特殊构筑商品店</x:v>
+        <x:v>灵感大王</x:v>
       </x:c>
       <x:c r="C37" t="str">
         <x:v>特殊店</x:v>
       </x:c>
       <x:c r="D37" t="str">
-        <x:v>特殊, 构筑</x:v>
+        <x:v>特殊, 精英奖励</x:v>
       </x:c>
       <x:c r="E37" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F37" t="str">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G37" t="str">
-        <x:v>事件价格</x:v>
+        <x:v>奖励规则</x:v>
       </x:c>
       <x:c r="H37" t="str">
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I37" t="str">
-        <x:v>复制、升阶等特殊构筑事件引用。</x:v>
+        <x:v>精英奖励和高压奖励引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
-        <x:v>elite_high</x:v>
+        <x:v>shop_store_37</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>精英高奖商品店</x:v>
+        <x:v>青牛精</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>特殊店</x:v>
+        <x:v>通用店</x:v>
       </x:c>
       <x:c r="D38" t="str">
-        <x:v>特殊, 精英奖励</x:v>
+        <x:v>通用, 夜市</x:v>
       </x:c>
       <x:c r="E38" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F38" t="str">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G38" t="str">
-        <x:v>奖励规则</x:v>
+        <x:v>标准价格</x:v>
       </x:c>
       <x:c r="H38" t="str">
         <x:v>正式</x:v>
       </x:c>
       <x:c r="I38" t="str">
-        <x:v>精英奖励和高压奖励引用。</x:v>
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>shop_store_38</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>太上老君</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>shop_store_39</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>如意真仙</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H40" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I40" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>shop_store_40</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>西梁女国国王</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I41" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>shop_store_41</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>蝎子精</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>shop_store_42</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>六耳猕猴</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>shop_store_43</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>如来佛祖</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>shop_store_44</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>牛魔王</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>shop_store_45</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>铁扇公主</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I46" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>shop_store_46</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>玉面狐狸</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>shop_store_47</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>各路神佛</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>shop_store_48</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>九头虫</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>shop_store_49</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>万圣老龙</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>shop_store_50</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>十八公</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>shop_store_51</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>孤直公</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I52" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>shop_store_52</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>凌空子</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I53" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>shop_store_53</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>拂云叟</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I54" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>shop_store_54</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>杏仙</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H55" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I55" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>shop_store_55</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>黄眉老佛</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I56" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>shop_store_56</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>蟒蛇精</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I57" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>shop_store_57</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>赛太岁</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>shop_store_58</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>蜘蛛精</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>shop_store_59</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>百眼魔君</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>shop_store_60</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>青狮</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>shop_store_61</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>白象</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>shop_store_62</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>大鹏金翅雕</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I63" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>shop_store_63</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>白鹿精</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I64" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>shop_store_64</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>白面狐狸</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>shop_store_65</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>金鼻白毛老鼠精</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I66" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>shop_store_66</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>灭法国国王</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>shop_store_67</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>南山大王</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I68" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>shop_store_68</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>凤仙郡郡侯</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>shop_store_69</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>玉帝</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>shop_store_70</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>黄狮精</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>shop_store_71</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>九灵元圣</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>shop_store_72</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>辟寒大王</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>shop_store_73</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>辟暑大王</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>shop_store_74</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>辟尘大王</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>shop_store_75</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>玉兔精</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>shop_store_76</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>寇洪及家人</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>shop_store_77</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>接引佛祖</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>shop_store_78</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>老鼋</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>通用店</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>通用, 夜市</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>基础商品店；大多数宠物可进入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>elem_无</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>凡兽铺</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>元素店</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>元素, 无</x:v>
+      </x:c>
+      <x:c r="E80" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F80" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>标准价格</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>正式</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>出售无元素宠物；保留正式路线和凡兽商品池兼容。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f85110635454e08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d82d641b644b2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>